<commit_message>
Update ARIMA and SARIMA to exact 5-year 80/20 split
</commit_message>
<xml_diff>
--- a/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
+++ b/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
@@ -657,31 +657,31 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>685.6274</v>
+        <v>351.7076</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>602.1919</v>
+        <v>295.9418</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>26.1277</v>
+        <v>13.0562</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>73.8723</v>
+        <v>86.9438</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-3.1643</v>
+        <v>-0.3415</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>47.4747</v>
+        <v>46.371</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.4693</v>
+        <v>0.4583</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.961</v>
+        <v>0.7521</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.6307</v>
+        <v>0.5696</v>
       </c>
     </row>
     <row r="3">
@@ -813,31 +813,31 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>683.0753999999999</v>
+        <v>355.1926</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>599.6116</v>
+        <v>299.7326</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>26.0201</v>
+        <v>13.2381</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>73.9799</v>
+        <v>86.7619</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>-3.1333</v>
+        <v>-0.3682</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>47.6768</v>
+        <v>46.371</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.4703</v>
+        <v>0.4588</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>0.961</v>
+        <v>0.7607</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.6316000000000001</v>
+        <v>0.5723</v>
       </c>
     </row>
     <row r="7">
@@ -891,31 +891,31 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>191.7399</v>
+        <v>173.0366</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>143.1735</v>
+        <v>118.1199</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>10.8691</v>
+        <v>7.2338</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>89.1309</v>
+        <v>92.7662</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.1089</v>
+        <v>-0.254</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>49.697</v>
+        <v>50.8065</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.4838</v>
+        <v>0.4839</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.6891</v>
+        <v>0.3782</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.5685</v>
+        <v>0.4245</v>
       </c>
     </row>
     <row r="9">
@@ -1047,31 +1047,31 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>192.3934</v>
+        <v>174.0953</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>143.9471</v>
+        <v>118.6982</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>10.9372</v>
+        <v>7.2626</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>89.0628</v>
+        <v>92.73739999999999</v>
       </c>
       <c r="G12" s="11" t="n">
-        <v>-0.1164</v>
+        <v>-0.2694</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>49.899</v>
+        <v>50.4032</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.4854</v>
+        <v>0.4778</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>0.6975</v>
+        <v>0.3613</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.5724</v>
+        <v>0.4115</v>
       </c>
     </row>
     <row r="13">
@@ -1125,31 +1125,31 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1095.6858</v>
+        <v>442.7054</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>956.8518</v>
+        <v>349.6725</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>12.7613</v>
+        <v>4.5433</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>87.23869999999999</v>
+        <v>95.4567</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-3.0117</v>
+        <v>-0.0069</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>50.9091</v>
+        <v>47.9839</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.5</v>
+        <v>0.4417</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.0329</v>
+        <v>0.4609</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0.0618</v>
+        <v>0.4511</v>
       </c>
     </row>
     <row r="15">
@@ -1281,31 +1281,31 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>1095.3127</v>
+        <v>442.0724</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>956.4059</v>
+        <v>349.4367</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>12.7551</v>
+        <v>4.546</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>87.2449</v>
+        <v>95.45399999999999</v>
       </c>
       <c r="G18" s="11" t="n">
-        <v>-3.009</v>
+        <v>-0.004</v>
       </c>
       <c r="H18" s="11" t="n">
-        <v>50.9091</v>
+        <v>47.9839</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.5</v>
+        <v>0.4426</v>
       </c>
       <c r="J18" s="11" t="n">
-        <v>0.0329</v>
+        <v>0.4696</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.0618</v>
+        <v>0.4557</v>
       </c>
     </row>
     <row r="19">
@@ -1359,31 +1359,31 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>430.257</v>
+        <v>221.8884</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>379.4956</v>
+        <v>173.6718</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>15.9381</v>
+        <v>6.6347</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>84.06189999999999</v>
+        <v>93.3653</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-1.1425</v>
+        <v>-0.3224</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>49.697</v>
+        <v>52.0161</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0.4937</v>
+        <v>0.5244</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.8033</v>
+        <v>0.3496</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>0.6115</v>
+        <v>0.4195</v>
       </c>
     </row>
     <row r="21">
@@ -1515,31 +1515,31 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>429.5524</v>
+        <v>214.4247</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>378.9045</v>
+        <v>168.6181</v>
       </c>
       <c r="E24" s="11" t="n">
-        <v>15.9119</v>
+        <v>6.4691</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>84.0881</v>
+        <v>93.5309</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>-1.1355</v>
+        <v>-0.235</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>49.899</v>
+        <v>51.2097</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>0.495</v>
+        <v>0.5111</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>0.8074</v>
+        <v>0.374</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.6137</v>
+        <v>0.4319</v>
       </c>
     </row>
     <row r="25">
@@ -1593,31 +1593,31 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>144.275</v>
+        <v>115.6991</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>118.0821</v>
+        <v>101.2427</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>10.5874</v>
+        <v>8.0176</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>89.4126</v>
+        <v>91.9824</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.9843</v>
+        <v>-0.4536</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>52.1212</v>
+        <v>50</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>0.5049</v>
+        <v>0.4923</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.8631</v>
+        <v>0.2602</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.6371</v>
+        <v>0.3404</v>
       </c>
     </row>
     <row r="27">
@@ -1749,31 +1749,31 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>141.8073</v>
+        <v>115.2568</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>115.766</v>
+        <v>100.8526</v>
       </c>
       <c r="E30" s="11" t="n">
-        <v>10.379</v>
+        <v>7.9898</v>
       </c>
       <c r="F30" s="11" t="n">
-        <v>89.621</v>
+        <v>92.0102</v>
       </c>
       <c r="G30" s="11" t="n">
-        <v>-0.917</v>
+        <v>-0.4425</v>
       </c>
       <c r="H30" s="11" t="n">
-        <v>51.9192</v>
+        <v>50</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>0.5037</v>
+        <v>0.4923</v>
       </c>
       <c r="J30" s="11" t="n">
-        <v>0.8506</v>
+        <v>0.2602</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.6327</v>
+        <v>0.3404</v>
       </c>
     </row>
     <row r="31">
@@ -1827,31 +1827,31 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>972.1457</v>
+        <v>1057.6268</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>772.0848</v>
+        <v>887.4546</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>8.6654</v>
+        <v>9.291700000000001</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>91.33459999999999</v>
+        <v>90.70829999999999</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.0211</v>
+        <v>-1.6353</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>51.5152</v>
+        <v>50.8065</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>0.5229</v>
+        <v>0.5517</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.6299</v>
+        <v>0.128</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0.5714</v>
+        <v>0.2078</v>
       </c>
     </row>
     <row r="33">
@@ -1983,31 +1983,31 @@
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>973.2443</v>
+        <v>1050.2834</v>
       </c>
       <c r="D36" s="11" t="n">
-        <v>773.8683</v>
+        <v>880.003</v>
       </c>
       <c r="E36" s="11" t="n">
-        <v>8.6919</v>
+        <v>9.2127</v>
       </c>
       <c r="F36" s="11" t="n">
-        <v>91.3081</v>
+        <v>90.7873</v>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-0.0234</v>
+        <v>-1.5988</v>
       </c>
       <c r="H36" s="11" t="n">
-        <v>51.5152</v>
+        <v>50.8065</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>0.5229</v>
+        <v>0.5517</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>0.6299</v>
+        <v>0.128</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.5714</v>
+        <v>0.2078</v>
       </c>
     </row>
     <row r="37">
@@ -2061,31 +2061,31 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>334.4322</v>
+        <v>150.0146</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>294.7112</v>
+        <v>112.5206</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>15.1089</v>
+        <v>6.1713</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>84.89109999999999</v>
+        <v>93.8287</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-3.3138</v>
+        <v>-0.2416</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>51.1111</v>
+        <v>52.8226</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.5833</v>
+        <v>0.4962</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0569</v>
+        <v>0.569</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.1037</v>
+        <v>0.5301</v>
       </c>
     </row>
     <row r="39">
@@ -2217,31 +2217,31 @@
         </is>
       </c>
       <c r="C42" s="11" t="n">
-        <v>333.6766</v>
+        <v>151.7565</v>
       </c>
       <c r="D42" s="11" t="n">
-        <v>293.927</v>
+        <v>112.876</v>
       </c>
       <c r="E42" s="11" t="n">
-        <v>15.0675</v>
+        <v>6.2009</v>
       </c>
       <c r="F42" s="11" t="n">
-        <v>84.9325</v>
+        <v>93.7991</v>
       </c>
       <c r="G42" s="11" t="n">
-        <v>-3.2944</v>
+        <v>-0.2706</v>
       </c>
       <c r="H42" s="11" t="n">
-        <v>51.1111</v>
+        <v>53.629</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>0.5833</v>
+        <v>0.5036</v>
       </c>
       <c r="J42" s="11" t="n">
-        <v>0.0569</v>
+        <v>0.5948</v>
       </c>
       <c r="K42" s="11" t="n">
-        <v>0.1037</v>
+        <v>0.5455</v>
       </c>
     </row>
     <row r="43">
@@ -2295,31 +2295,31 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>205.6415</v>
+        <v>69.41419999999999</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>175.0832</v>
+        <v>57.1309</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>18.8612</v>
+        <v>5.8722</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>81.1388</v>
+        <v>94.12779999999999</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>-1.8994</v>
+        <v>-0.2766</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>49.899</v>
+        <v>52.8226</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.5443</v>
+        <v>0.5926</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.1686</v>
+        <v>0.3636</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2575</v>
+        <v>0.4507</v>
       </c>
     </row>
     <row r="45">
@@ -2451,31 +2451,31 @@
         </is>
       </c>
       <c r="C48" s="11" t="n">
-        <v>204.556</v>
+        <v>69.6053</v>
       </c>
       <c r="D48" s="11" t="n">
-        <v>174.1716</v>
+        <v>57.2697</v>
       </c>
       <c r="E48" s="11" t="n">
-        <v>18.7667</v>
+        <v>5.8847</v>
       </c>
       <c r="F48" s="11" t="n">
-        <v>81.2333</v>
+        <v>94.1153</v>
       </c>
       <c r="G48" s="11" t="n">
-        <v>-1.8689</v>
+        <v>-0.2837</v>
       </c>
       <c r="H48" s="11" t="n">
-        <v>50.101</v>
+        <v>53.2258</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>0.5488</v>
+        <v>0.5976</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>0.1765</v>
+        <v>0.3712</v>
       </c>
       <c r="K48" s="11" t="n">
-        <v>0.2671</v>
+        <v>0.4579</v>
       </c>
     </row>
     <row r="49">
@@ -2529,31 +2529,31 @@
         </is>
       </c>
       <c r="C50" s="3" t="n">
-        <v>429.0361</v>
+        <v>125.2284</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>385.7323</v>
+        <v>109.2805</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>20.5293</v>
+        <v>5.7588</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>79.47069999999999</v>
+        <v>94.24120000000001</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-4.2164</v>
+        <v>-0.514</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>49.0909</v>
+        <v>52.0161</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>1</v>
+        <v>0.5083</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0.004</v>
+        <v>0.7541</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.6073</v>
       </c>
     </row>
     <row r="51">
@@ -2685,31 +2685,31 @@
         </is>
       </c>
       <c r="C54" s="11" t="n">
-        <v>428.6824</v>
+        <v>129.0358</v>
       </c>
       <c r="D54" s="11" t="n">
-        <v>385.3411</v>
+        <v>112.2982</v>
       </c>
       <c r="E54" s="11" t="n">
-        <v>20.5074</v>
+        <v>5.9267</v>
       </c>
       <c r="F54" s="11" t="n">
-        <v>79.4926</v>
+        <v>94.0733</v>
       </c>
       <c r="G54" s="11" t="n">
-        <v>-4.2078</v>
+        <v>-0.6074000000000001</v>
       </c>
       <c r="H54" s="11" t="n">
-        <v>49.0909</v>
+        <v>50.8065</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>0.004</v>
+        <v>0.7705</v>
       </c>
       <c r="K54" s="11" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.6065</v>
       </c>
     </row>
     <row r="55">
@@ -2763,31 +2763,31 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>50.8322</v>
+        <v>28.515</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>42.1697</v>
+        <v>24.9061</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>13.1185</v>
+        <v>7.666</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>86.8815</v>
+        <v>92.334</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>-1.1148</v>
+        <v>-0.0064</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>53.7374</v>
+        <v>47.1774</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>0.5571</v>
+        <v>0.4258</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>0.1646</v>
+        <v>0.6111</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>0.2541</v>
+        <v>0.5019</v>
       </c>
     </row>
     <row r="57">
@@ -2919,31 +2919,31 @@
         </is>
       </c>
       <c r="C60" s="11" t="n">
-        <v>51.022</v>
+        <v>29.3565</v>
       </c>
       <c r="D60" s="11" t="n">
-        <v>42.3548</v>
+        <v>26.1926</v>
       </c>
       <c r="E60" s="11" t="n">
-        <v>13.1749</v>
+        <v>8.178699999999999</v>
       </c>
       <c r="F60" s="11" t="n">
-        <v>86.82510000000001</v>
+        <v>91.82129999999999</v>
       </c>
       <c r="G60" s="11" t="n">
-        <v>-1.1306</v>
+        <v>-0.0667</v>
       </c>
       <c r="H60" s="11" t="n">
-        <v>53.5354</v>
+        <v>45.9677</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>0.5507</v>
+        <v>0.4177</v>
       </c>
       <c r="J60" s="11" t="n">
-        <v>0.1603</v>
+        <v>0.6111</v>
       </c>
       <c r="K60" s="11" t="n">
-        <v>0.2484</v>
+        <v>0.4962</v>
       </c>
     </row>
     <row r="61">
@@ -2997,31 +2997,31 @@
         </is>
       </c>
       <c r="C62" s="3" t="n">
-        <v>444.8542</v>
+        <v>297.95</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>371.6456</v>
+        <v>231.5737</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>6.9262</v>
+        <v>4.1492</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>93.07380000000001</v>
+        <v>95.85080000000001</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>-0.0001</v>
+        <v>-0.0423</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>51.9192</v>
+        <v>57.2581</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>0.5588</v>
+        <v>0.5946</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>0.4351</v>
+        <v>0.5197000000000001</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>0.4893</v>
+        <v>0.5546</v>
       </c>
     </row>
     <row r="63">
@@ -3153,31 +3153,31 @@
         </is>
       </c>
       <c r="C66" s="11" t="n">
-        <v>444.9467</v>
+        <v>297.7072</v>
       </c>
       <c r="D66" s="11" t="n">
-        <v>372.8352</v>
+        <v>231.9432</v>
       </c>
       <c r="E66" s="11" t="n">
-        <v>6.9388</v>
+        <v>4.1546</v>
       </c>
       <c r="F66" s="11" t="n">
-        <v>93.0612</v>
+        <v>95.8454</v>
       </c>
       <c r="G66" s="11" t="n">
-        <v>-0.0005</v>
+        <v>-0.0406</v>
       </c>
       <c r="H66" s="11" t="n">
-        <v>51.7172</v>
+        <v>55.6452</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>0.5567</v>
+        <v>0.5752</v>
       </c>
       <c r="J66" s="11" t="n">
-        <v>0.4313</v>
+        <v>0.5118</v>
       </c>
       <c r="K66" s="11" t="n">
-        <v>0.486</v>
+        <v>0.5417</v>
       </c>
     </row>
     <row r="67">
@@ -3231,31 +3231,31 @@
         </is>
       </c>
       <c r="C68" s="3" t="n">
-        <v>94.256</v>
+        <v>129.4961</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>69.6211</v>
+        <v>96.3652</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>4.9596</v>
+        <v>7.2386</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>95.04040000000001</v>
+        <v>92.76139999999999</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>-0.0181</v>
+        <v>-0.4374</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>51.7172</v>
+        <v>50.8065</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>0.525</v>
+        <v>0.503</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>0.502</v>
+        <v>0.6829</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>0.5132</v>
+        <v>0.5793</v>
       </c>
     </row>
     <row r="69">
@@ -3387,31 +3387,31 @@
         </is>
       </c>
       <c r="C72" s="11" t="n">
-        <v>94.26130000000001</v>
+        <v>129.8967</v>
       </c>
       <c r="D72" s="11" t="n">
-        <v>69.62569999999999</v>
+        <v>96.61360000000001</v>
       </c>
       <c r="E72" s="11" t="n">
-        <v>4.96</v>
+        <v>7.2587</v>
       </c>
       <c r="F72" s="11" t="n">
-        <v>95.04000000000001</v>
+        <v>92.7413</v>
       </c>
       <c r="G72" s="11" t="n">
-        <v>-0.0183</v>
+        <v>-0.4463</v>
       </c>
       <c r="H72" s="11" t="n">
-        <v>51.5152</v>
+        <v>50.4032</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>0.5228</v>
+        <v>0.5</v>
       </c>
       <c r="J72" s="11" t="n">
-        <v>0.502</v>
+        <v>0.6992</v>
       </c>
       <c r="K72" s="11" t="n">
-        <v>0.5122</v>
+        <v>0.5831</v>
       </c>
     </row>
     <row r="73">
@@ -3465,31 +3465,31 @@
         </is>
       </c>
       <c r="C74" s="3" t="n">
-        <v>54.1463</v>
+        <v>62.8312</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46.3006</v>
+        <v>49.4396</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>12.3574</v>
+        <v>11.313</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>87.6426</v>
+        <v>88.687</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>-0.7487</v>
+        <v>-1.5486</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>54.7475</v>
+        <v>49.5968</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>0.5395</v>
+        <v>0.6</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>0.7579</v>
+        <v>0.0703</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>0.6304</v>
+        <v>0.1259</v>
       </c>
     </row>
     <row r="75">
@@ -3621,31 +3621,31 @@
         </is>
       </c>
       <c r="C78" s="11" t="n">
-        <v>54.4781</v>
+        <v>62.8951</v>
       </c>
       <c r="D78" s="11" t="n">
-        <v>46.5252</v>
+        <v>49.5118</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>12.4233</v>
+        <v>11.3305</v>
       </c>
       <c r="F78" s="11" t="n">
-        <v>87.5767</v>
+        <v>88.6695</v>
       </c>
       <c r="G78" s="11" t="n">
-        <v>-0.7702</v>
+        <v>-1.5538</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>55.1515</v>
+        <v>49.5968</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0.5424</v>
+        <v>0.6</v>
       </c>
       <c r="J78" s="11" t="n">
-        <v>0.7619</v>
+        <v>0.0703</v>
       </c>
       <c r="K78" s="11" t="n">
-        <v>0.6337</v>
+        <v>0.1259</v>
       </c>
     </row>
     <row r="79">
@@ -3699,31 +3699,31 @@
         </is>
       </c>
       <c r="C80" s="3" t="n">
-        <v>1728.4874</v>
+        <v>558.8559</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>1638.302</v>
+        <v>480.061</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>26.3634</v>
+        <v>7.7458</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>73.6366</v>
+        <v>92.2542</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>-8.8348</v>
+        <v>-2.694</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>48.8889</v>
+        <v>50.8065</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>0</v>
+        <v>0.4958</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>0</v>
+        <v>0.9917</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>0</v>
+        <v>0.6611</v>
       </c>
     </row>
     <row r="81">
@@ -3855,31 +3855,31 @@
         </is>
       </c>
       <c r="C84" s="11" t="n">
-        <v>1737.8542</v>
+        <v>582.7045000000001</v>
       </c>
       <c r="D84" s="11" t="n">
-        <v>1648.0764</v>
+        <v>506.1231</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>26.5255</v>
+        <v>8.1571</v>
       </c>
       <c r="F84" s="11" t="n">
-        <v>73.47450000000001</v>
+        <v>91.8429</v>
       </c>
       <c r="G84" s="11" t="n">
-        <v>-8.941700000000001</v>
+        <v>-3.016</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>48.8889</v>
+        <v>50</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0</v>
+        <v>0.4917</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>0</v>
+        <v>0.9917</v>
       </c>
       <c r="K84" s="11" t="n">
-        <v>0</v>
+        <v>0.6575</v>
       </c>
     </row>
     <row r="85">
@@ -3933,31 +3933,31 @@
         </is>
       </c>
       <c r="C86" s="3" t="n">
-        <v>75.0754</v>
+        <v>55.8888</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>59.1507</v>
+        <v>46.281</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>4.8434</v>
+        <v>3.7253</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>95.1566</v>
+        <v>96.2747</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>-0.3377</v>
+        <v>-0.9081</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>56.3636</v>
+        <v>56.8548</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>0.5481</v>
+        <v>0.5433</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>0.755</v>
+        <v>0.904</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>0.6351</v>
+        <v>0.6787</v>
       </c>
     </row>
     <row r="87">
@@ -4089,31 +4089,31 @@
         </is>
       </c>
       <c r="C90" s="11" t="n">
-        <v>74.3437</v>
+        <v>53.9433</v>
       </c>
       <c r="D90" s="11" t="n">
-        <v>58.5956</v>
+        <v>44.4186</v>
       </c>
       <c r="E90" s="11" t="n">
-        <v>4.7952</v>
+        <v>3.5744</v>
       </c>
       <c r="F90" s="11" t="n">
-        <v>95.20480000000001</v>
+        <v>96.4256</v>
       </c>
       <c r="G90" s="11" t="n">
-        <v>-0.3118</v>
+        <v>-0.7775</v>
       </c>
       <c r="H90" s="11" t="n">
-        <v>56.1616</v>
+        <v>57.2581</v>
       </c>
       <c r="I90" s="11" t="n">
-        <v>0.5473</v>
+        <v>0.5468</v>
       </c>
       <c r="J90" s="11" t="n">
-        <v>0.743</v>
+        <v>0.888</v>
       </c>
       <c r="K90" s="11" t="n">
-        <v>0.6303</v>
+        <v>0.6768</v>
       </c>
     </row>
     <row r="91">
@@ -4167,31 +4167,31 @@
         </is>
       </c>
       <c r="C92" s="3" t="n">
-        <v>1657.2338</v>
+        <v>1465.9442</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>1263.3543</v>
+        <v>1346.6738</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>18.5996</v>
+        <v>18.7539</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>81.4004</v>
+        <v>81.2461</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>-1.3286</v>
+        <v>-4.5</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>50.303</v>
+        <v>49.1935</v>
       </c>
       <c r="I92" s="3" t="n">
-        <v>0.5385</v>
+        <v>0.5556</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>0.0843</v>
+        <v>0.0781</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>0.1458</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="93">
@@ -4323,31 +4323,31 @@
         </is>
       </c>
       <c r="C96" s="11" t="n">
-        <v>1658.9111</v>
+        <v>1460.6877</v>
       </c>
       <c r="D96" s="11" t="n">
-        <v>1265.2398</v>
+        <v>1341.661</v>
       </c>
       <c r="E96" s="11" t="n">
-        <v>18.6308</v>
+        <v>18.6839</v>
       </c>
       <c r="F96" s="11" t="n">
-        <v>81.36920000000001</v>
+        <v>81.31610000000001</v>
       </c>
       <c r="G96" s="11" t="n">
-        <v>-1.3333</v>
+        <v>-4.4606</v>
       </c>
       <c r="H96" s="11" t="n">
-        <v>50.5051</v>
+        <v>48.7903</v>
       </c>
       <c r="I96" s="11" t="n">
-        <v>0.5526</v>
+        <v>0.5263</v>
       </c>
       <c r="J96" s="11" t="n">
-        <v>0.0843</v>
+        <v>0.0781</v>
       </c>
       <c r="K96" s="11" t="n">
-        <v>0.1463</v>
+        <v>0.1361</v>
       </c>
     </row>
     <row r="97">
@@ -4401,31 +4401,31 @@
         </is>
       </c>
       <c r="C98" s="3" t="n">
-        <v>179.1919</v>
+        <v>155.1122</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>131.2935</v>
+        <v>105.0373</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>4.8977</v>
+        <v>3.5673</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>95.1023</v>
+        <v>96.4327</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>-0.0115</v>
+        <v>-0.2241</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>53.9394</v>
+        <v>54.8387</v>
       </c>
       <c r="I98" s="3" t="n">
-        <v>0.5269</v>
+        <v>0.5976</v>
       </c>
       <c r="J98" s="3" t="n">
-        <v>0.5661</v>
+        <v>0.3828</v>
       </c>
       <c r="K98" s="3" t="n">
-        <v>0.5458</v>
+        <v>0.4667</v>
       </c>
     </row>
     <row r="99">
@@ -4557,31 +4557,31 @@
         </is>
       </c>
       <c r="C102" s="11" t="n">
-        <v>179.8849</v>
+        <v>154.5579</v>
       </c>
       <c r="D102" s="11" t="n">
-        <v>131.7815</v>
+        <v>104.6118</v>
       </c>
       <c r="E102" s="11" t="n">
-        <v>4.9254</v>
+        <v>3.5536</v>
       </c>
       <c r="F102" s="11" t="n">
-        <v>95.0746</v>
+        <v>96.4464</v>
       </c>
       <c r="G102" s="11" t="n">
-        <v>-0.0193</v>
+        <v>-0.2154</v>
       </c>
       <c r="H102" s="11" t="n">
-        <v>53.5354</v>
+        <v>55.2419</v>
       </c>
       <c r="I102" s="11" t="n">
-        <v>0.5216</v>
+        <v>0.6024</v>
       </c>
       <c r="J102" s="11" t="n">
-        <v>0.5992</v>
+        <v>0.3906</v>
       </c>
       <c r="K102" s="11" t="n">
-        <v>0.5577</v>
+        <v>0.4739</v>
       </c>
     </row>
     <row r="103">
@@ -4635,31 +4635,31 @@
         </is>
       </c>
       <c r="C104" s="3" t="n">
-        <v>202.9022</v>
+        <v>282.0651</v>
       </c>
       <c r="D104" s="3" t="n">
-        <v>169.0958</v>
+        <v>231.879</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>11.0563</v>
+        <v>18.0914</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>88.94370000000001</v>
+        <v>81.90860000000001</v>
       </c>
       <c r="G104" s="3" t="n">
-        <v>-0.2931</v>
+        <v>-1.9292</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>52.1212</v>
+        <v>47.1774</v>
       </c>
       <c r="I104" s="3" t="n">
-        <v>0.5039</v>
+        <v>0.4681</v>
       </c>
       <c r="J104" s="3" t="n">
-        <v>0.2731</v>
+        <v>0.9483</v>
       </c>
       <c r="K104" s="3" t="n">
-        <v>0.3542</v>
+        <v>0.6268</v>
       </c>
     </row>
     <row r="105">
@@ -4791,31 +4791,31 @@
         </is>
       </c>
       <c r="C108" s="11" t="n">
-        <v>201.6731</v>
+        <v>281.1373</v>
       </c>
       <c r="D108" s="11" t="n">
-        <v>167.8917</v>
+        <v>230.9243</v>
       </c>
       <c r="E108" s="11" t="n">
-        <v>10.9918</v>
+        <v>18.0204</v>
       </c>
       <c r="F108" s="11" t="n">
-        <v>89.0082</v>
+        <v>81.9796</v>
       </c>
       <c r="G108" s="11" t="n">
-        <v>-0.2775</v>
+        <v>-1.9099</v>
       </c>
       <c r="H108" s="11" t="n">
-        <v>51.9192</v>
+        <v>47.1774</v>
       </c>
       <c r="I108" s="11" t="n">
-        <v>0.5</v>
+        <v>0.4678</v>
       </c>
       <c r="J108" s="11" t="n">
-        <v>0.2731</v>
+        <v>0.9397</v>
       </c>
       <c r="K108" s="11" t="n">
-        <v>0.3533</v>
+        <v>0.6246</v>
       </c>
     </row>
     <row r="109">
@@ -4869,31 +4869,31 @@
         </is>
       </c>
       <c r="C110" s="3" t="n">
-        <v>114.7874</v>
+        <v>122.2779</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>92.37990000000001</v>
+        <v>85.07389999999999</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>9.9764</v>
+        <v>10.7113</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>90.0236</v>
+        <v>89.28870000000001</v>
       </c>
       <c r="G110" s="3" t="n">
-        <v>-1.117</v>
+        <v>-0.7717000000000001</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>53.1313</v>
+        <v>47.9839</v>
       </c>
       <c r="I110" s="3" t="n">
-        <v>0.5393</v>
+        <v>0.4432</v>
       </c>
       <c r="J110" s="3" t="n">
-        <v>0.2008</v>
+        <v>0.7593</v>
       </c>
       <c r="K110" s="3" t="n">
-        <v>0.2927</v>
+        <v>0.5597</v>
       </c>
     </row>
     <row r="111">
@@ -5025,31 +5025,31 @@
         </is>
       </c>
       <c r="C114" s="11" t="n">
-        <v>113.2311</v>
+        <v>122.0621</v>
       </c>
       <c r="D114" s="11" t="n">
-        <v>91.00320000000001</v>
+        <v>84.9119</v>
       </c>
       <c r="E114" s="11" t="n">
-        <v>9.829700000000001</v>
+        <v>10.6911</v>
       </c>
       <c r="F114" s="11" t="n">
-        <v>90.1703</v>
+        <v>89.30889999999999</v>
       </c>
       <c r="G114" s="11" t="n">
-        <v>-1.0599</v>
+        <v>-0.7654</v>
       </c>
       <c r="H114" s="11" t="n">
-        <v>53.3333</v>
+        <v>47.9839</v>
       </c>
       <c r="I114" s="11" t="n">
-        <v>0.5435</v>
+        <v>0.4426</v>
       </c>
       <c r="J114" s="11" t="n">
-        <v>0.2092</v>
+        <v>0.75</v>
       </c>
       <c r="K114" s="11" t="n">
-        <v>0.3021</v>
+        <v>0.5567</v>
       </c>
     </row>
     <row r="115">
@@ -5103,31 +5103,31 @@
         </is>
       </c>
       <c r="C116" s="3" t="n">
-        <v>98.825</v>
+        <v>114.9212</v>
       </c>
       <c r="D116" s="3" t="n">
-        <v>82.6495</v>
+        <v>86.7132</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>11.3238</v>
+        <v>13.8242</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>88.67619999999999</v>
+        <v>86.1758</v>
       </c>
       <c r="G116" s="3" t="n">
-        <v>-1.2302</v>
+        <v>-1.3076</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>52.1212</v>
+        <v>43.9516</v>
       </c>
       <c r="I116" s="3" t="n">
-        <v>0.4952</v>
+        <v>0.4362</v>
       </c>
       <c r="J116" s="3" t="n">
-        <v>0.2203</v>
+        <v>0.9815</v>
       </c>
       <c r="K116" s="3" t="n">
-        <v>0.305</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="117">
@@ -5259,31 +5259,31 @@
         </is>
       </c>
       <c r="C120" s="11" t="n">
-        <v>122.3946</v>
+        <v>114.5254</v>
       </c>
       <c r="D120" s="11" t="n">
-        <v>103.5753</v>
+        <v>86.21120000000001</v>
       </c>
       <c r="E120" s="11" t="n">
-        <v>14.1695</v>
+        <v>13.7511</v>
       </c>
       <c r="F120" s="11" t="n">
-        <v>85.8305</v>
+        <v>86.24890000000001</v>
       </c>
       <c r="G120" s="11" t="n">
-        <v>-2.4209</v>
+        <v>-1.2917</v>
       </c>
       <c r="H120" s="11" t="n">
-        <v>51.9192</v>
+        <v>43.5484</v>
       </c>
       <c r="I120" s="11" t="n">
-        <v>0.4545</v>
+        <v>0.4333</v>
       </c>
       <c r="J120" s="11" t="n">
-        <v>0.0424</v>
+        <v>0.963</v>
       </c>
       <c r="K120" s="11" t="n">
-        <v>0.0775</v>
+        <v>0.5977</v>
       </c>
     </row>
     <row r="121">
@@ -5337,31 +5337,31 @@
         </is>
       </c>
       <c r="C122" s="3" t="n">
-        <v>829.3754</v>
+        <v>1169.3135</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>641.3952</v>
+        <v>1077.7915</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>15.2605</v>
+        <v>19.9371</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>84.73950000000001</v>
+        <v>80.0629</v>
       </c>
       <c r="G122" s="3" t="n">
-        <v>-0.3815</v>
+        <v>-5.5655</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>51.9192</v>
+        <v>49.5968</v>
       </c>
       <c r="I122" s="3" t="n">
-        <v>0.5165</v>
+        <v>0.8</v>
       </c>
       <c r="J122" s="3" t="n">
-        <v>0.6908</v>
+        <v>0.0312</v>
       </c>
       <c r="K122" s="3" t="n">
-        <v>0.5911</v>
+        <v>0.0602</v>
       </c>
     </row>
     <row r="123">
@@ -5493,31 +5493,31 @@
         </is>
       </c>
       <c r="C126" s="11" t="n">
-        <v>832.6152</v>
+        <v>1174.0794</v>
       </c>
       <c r="D126" s="11" t="n">
-        <v>643.4959</v>
+        <v>1082.849</v>
       </c>
       <c r="E126" s="11" t="n">
-        <v>15.3186</v>
+        <v>20.0338</v>
       </c>
       <c r="F126" s="11" t="n">
-        <v>84.6814</v>
+        <v>79.9662</v>
       </c>
       <c r="G126" s="11" t="n">
-        <v>-0.3924</v>
+        <v>-5.6191</v>
       </c>
       <c r="H126" s="11" t="n">
-        <v>51.5152</v>
+        <v>49.5968</v>
       </c>
       <c r="I126" s="11" t="n">
-        <v>0.5134</v>
+        <v>1</v>
       </c>
       <c r="J126" s="11" t="n">
-        <v>0.6908</v>
+        <v>0.0234</v>
       </c>
       <c r="K126" s="11" t="n">
-        <v>0.589</v>
+        <v>0.0458</v>
       </c>
     </row>
     <row r="127">
@@ -5571,31 +5571,31 @@
         </is>
       </c>
       <c r="C128" s="3" t="n">
-        <v>162.8584</v>
+        <v>229.5577</v>
       </c>
       <c r="D128" s="3" t="n">
-        <v>118.3851</v>
+        <v>191.3158</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>13.91</v>
+        <v>20.1335</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>86.09</v>
+        <v>79.8665</v>
       </c>
       <c r="G128" s="3" t="n">
-        <v>-0.196</v>
+        <v>-2.106</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>48.6869</v>
+        <v>44.7581</v>
       </c>
       <c r="I128" s="3" t="n">
-        <v>0.5323</v>
+        <v>0.5455</v>
       </c>
       <c r="J128" s="3" t="n">
-        <v>0.4889</v>
+        <v>0.0863</v>
       </c>
       <c r="K128" s="3" t="n">
-        <v>0.5097</v>
+        <v>0.1491</v>
       </c>
     </row>
     <row r="129">
@@ -5727,31 +5727,31 @@
         </is>
       </c>
       <c r="C132" s="11" t="n">
-        <v>162.6333</v>
+        <v>228.7028</v>
       </c>
       <c r="D132" s="11" t="n">
-        <v>118.3831</v>
+        <v>190.4576</v>
       </c>
       <c r="E132" s="11" t="n">
-        <v>13.9208</v>
+        <v>20.039</v>
       </c>
       <c r="F132" s="11" t="n">
-        <v>86.0792</v>
+        <v>79.961</v>
       </c>
       <c r="G132" s="11" t="n">
-        <v>-0.1926</v>
+        <v>-2.0829</v>
       </c>
       <c r="H132" s="11" t="n">
-        <v>48.6869</v>
+        <v>43.9516</v>
       </c>
       <c r="I132" s="11" t="n">
-        <v>0.5323</v>
+        <v>0.5</v>
       </c>
       <c r="J132" s="11" t="n">
-        <v>0.4889</v>
+        <v>0.0863</v>
       </c>
       <c r="K132" s="11" t="n">
-        <v>0.5097</v>
+        <v>0.1472</v>
       </c>
     </row>
     <row r="133">
@@ -5805,31 +5805,31 @@
         </is>
       </c>
       <c r="C134" s="3" t="n">
-        <v>216.7168</v>
+        <v>152.9717</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>187.6627</v>
+        <v>126.6005</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>8.1579</v>
+        <v>5.5434</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>91.8421</v>
+        <v>94.45659999999999</v>
       </c>
       <c r="G134" s="3" t="n">
-        <v>-0.4609</v>
+        <v>-0.0357</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>49.4949</v>
+        <v>53.629</v>
       </c>
       <c r="I134" s="3" t="n">
-        <v>0.4805</v>
+        <v>0.4848</v>
       </c>
       <c r="J134" s="3" t="n">
-        <v>0.7872</v>
+        <v>0.5766</v>
       </c>
       <c r="K134" s="3" t="n">
-        <v>0.5968</v>
+        <v>0.5266999999999999</v>
       </c>
     </row>
     <row r="135">
@@ -5961,31 +5961,31 @@
         </is>
       </c>
       <c r="C138" s="11" t="n">
-        <v>214.375</v>
+        <v>154.0133</v>
       </c>
       <c r="D138" s="11" t="n">
-        <v>185.3282</v>
+        <v>127.0354</v>
       </c>
       <c r="E138" s="11" t="n">
-        <v>8.0503</v>
+        <v>5.5739</v>
       </c>
       <c r="F138" s="11" t="n">
-        <v>91.94970000000001</v>
+        <v>94.42610000000001</v>
       </c>
       <c r="G138" s="11" t="n">
-        <v>-0.4295</v>
+        <v>-0.0498</v>
       </c>
       <c r="H138" s="11" t="n">
-        <v>49.2929</v>
+        <v>53.629</v>
       </c>
       <c r="I138" s="11" t="n">
-        <v>0.4791</v>
+        <v>0.4853</v>
       </c>
       <c r="J138" s="11" t="n">
-        <v>0.7786999999999999</v>
+        <v>0.5946</v>
       </c>
       <c r="K138" s="11" t="n">
-        <v>0.5931999999999999</v>
+        <v>0.5344</v>
       </c>
     </row>
     <row r="139">
@@ -6039,31 +6039,31 @@
         </is>
       </c>
       <c r="C140" s="3" t="n">
-        <v>122.7822</v>
+        <v>89.4136</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>100.6251</v>
+        <v>68.98779999999999</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>7.3162</v>
+        <v>5.273</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>92.68380000000001</v>
+        <v>94.727</v>
       </c>
       <c r="G140" s="3" t="n">
-        <v>-1.2417</v>
+        <v>-1.0551</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>53.5354</v>
+        <v>50.4032</v>
       </c>
       <c r="I140" s="3" t="n">
-        <v>0.5974</v>
+        <v>0.4771</v>
       </c>
       <c r="J140" s="3" t="n">
-        <v>0.1878</v>
+        <v>0.9204</v>
       </c>
       <c r="K140" s="3" t="n">
-        <v>0.2857</v>
+        <v>0.6284</v>
       </c>
     </row>
     <row r="141">
@@ -6195,31 +6195,31 @@
         </is>
       </c>
       <c r="C144" s="11" t="n">
-        <v>124.4879</v>
+        <v>89.37009999999999</v>
       </c>
       <c r="D144" s="11" t="n">
-        <v>102.1907</v>
+        <v>68.9427</v>
       </c>
       <c r="E144" s="11" t="n">
-        <v>7.4296</v>
+        <v>5.2696</v>
       </c>
       <c r="F144" s="11" t="n">
-        <v>92.57040000000001</v>
+        <v>94.7304</v>
       </c>
       <c r="G144" s="11" t="n">
-        <v>-1.3044</v>
+        <v>-1.0531</v>
       </c>
       <c r="H144" s="11" t="n">
-        <v>53.7374</v>
+        <v>50.4032</v>
       </c>
       <c r="I144" s="11" t="n">
-        <v>0.6081</v>
+        <v>0.4771</v>
       </c>
       <c r="J144" s="11" t="n">
-        <v>0.1837</v>
+        <v>0.9204</v>
       </c>
       <c r="K144" s="11" t="n">
-        <v>0.2821</v>
+        <v>0.6284</v>
       </c>
     </row>
     <row r="145">
@@ -6273,31 +6273,31 @@
         </is>
       </c>
       <c r="C146" s="3" t="n">
-        <v>526.3553000000001</v>
+        <v>67.2782</v>
       </c>
       <c r="D146" s="3" t="n">
-        <v>484.6661</v>
+        <v>57.1518</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>57.2797</v>
+        <v>6.8829</v>
       </c>
       <c r="F146" s="3" t="n">
-        <v>42.7203</v>
+        <v>93.11709999999999</v>
       </c>
       <c r="G146" s="3" t="n">
-        <v>-5.3138</v>
+        <v>-0.0039</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>49.899</v>
+        <v>51.6129</v>
       </c>
       <c r="I146" s="3" t="n">
-        <v>0.4947</v>
+        <v>0.5116000000000001</v>
       </c>
       <c r="J146" s="3" t="n">
-        <v>0.963</v>
+        <v>0.5366</v>
       </c>
       <c r="K146" s="3" t="n">
-        <v>0.6536</v>
+        <v>0.5238</v>
       </c>
     </row>
     <row r="147">
@@ -6429,31 +6429,31 @@
         </is>
       </c>
       <c r="C150" s="11" t="n">
-        <v>524.6367</v>
+        <v>67.2928</v>
       </c>
       <c r="D150" s="11" t="n">
-        <v>483.1254</v>
+        <v>57.165</v>
       </c>
       <c r="E150" s="11" t="n">
-        <v>57.0968</v>
+        <v>6.8861</v>
       </c>
       <c r="F150" s="11" t="n">
-        <v>42.9032</v>
+        <v>93.1139</v>
       </c>
       <c r="G150" s="11" t="n">
-        <v>-5.2726</v>
+        <v>-0.0043</v>
       </c>
       <c r="H150" s="11" t="n">
-        <v>49.899</v>
+        <v>51.2097</v>
       </c>
       <c r="I150" s="11" t="n">
-        <v>0.4947</v>
+        <v>0.5077</v>
       </c>
       <c r="J150" s="11" t="n">
-        <v>0.9671</v>
+        <v>0.5366</v>
       </c>
       <c r="K150" s="11" t="n">
-        <v>0.6546</v>
+        <v>0.5217000000000001</v>
       </c>
     </row>
     <row r="151">
@@ -6507,31 +6507,31 @@
         </is>
       </c>
       <c r="C152" s="3" t="n">
-        <v>221.0604</v>
+        <v>255.7696</v>
       </c>
       <c r="D152" s="3" t="n">
-        <v>179.9819</v>
+        <v>201.0458</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>12.7394</v>
+        <v>16.3787</v>
       </c>
       <c r="F152" s="3" t="n">
-        <v>87.2606</v>
+        <v>83.62130000000001</v>
       </c>
       <c r="G152" s="3" t="n">
-        <v>-0.0215</v>
+        <v>-1.2447</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>48.4848</v>
+        <v>47.1774</v>
       </c>
       <c r="I152" s="3" t="n">
-        <v>0.4764</v>
+        <v>0.446</v>
       </c>
       <c r="J152" s="3" t="n">
-        <v>0.5413</v>
+        <v>0.8796</v>
       </c>
       <c r="K152" s="3" t="n">
-        <v>0.5068</v>
+        <v>0.5919</v>
       </c>
     </row>
     <row r="153">
@@ -6663,31 +6663,31 @@
         </is>
       </c>
       <c r="C156" s="11" t="n">
-        <v>221.9083</v>
+        <v>256.4969</v>
       </c>
       <c r="D156" s="11" t="n">
-        <v>180.6694</v>
+        <v>201.748</v>
       </c>
       <c r="E156" s="11" t="n">
-        <v>12.8266</v>
+        <v>16.4337</v>
       </c>
       <c r="F156" s="11" t="n">
-        <v>87.1734</v>
+        <v>83.5663</v>
       </c>
       <c r="G156" s="11" t="n">
-        <v>-0.0293</v>
+        <v>-1.2575</v>
       </c>
       <c r="H156" s="11" t="n">
-        <v>49.2929</v>
+        <v>47.5806</v>
       </c>
       <c r="I156" s="11" t="n">
-        <v>0.4839</v>
+        <v>0.4486</v>
       </c>
       <c r="J156" s="11" t="n">
-        <v>0.5579</v>
+        <v>0.8889</v>
       </c>
       <c r="K156" s="11" t="n">
-        <v>0.5182</v>
+        <v>0.5963000000000001</v>
       </c>
     </row>
     <row r="157">
@@ -6741,31 +6741,31 @@
         </is>
       </c>
       <c r="C158" s="3" t="n">
-        <v>55.6555</v>
+        <v>70.0489</v>
       </c>
       <c r="D158" s="3" t="n">
-        <v>39.5293</v>
+        <v>53.5117</v>
       </c>
       <c r="E158" s="3" t="n">
-        <v>11.9838</v>
+        <v>17.6491</v>
       </c>
       <c r="F158" s="3" t="n">
-        <v>88.0162</v>
+        <v>82.3509</v>
       </c>
       <c r="G158" s="3" t="n">
-        <v>-0.2047</v>
+        <v>-1.3413</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>51.3131</v>
+        <v>46.371</v>
       </c>
       <c r="I158" s="3" t="n">
-        <v>0.4832</v>
+        <v>0.4537</v>
       </c>
       <c r="J158" s="3" t="n">
-        <v>0.6870000000000001</v>
+        <v>0.9196</v>
       </c>
       <c r="K158" s="3" t="n">
-        <v>0.5673</v>
+        <v>0.6077</v>
       </c>
     </row>
     <row r="159">
@@ -6897,31 +6897,31 @@
         </is>
       </c>
       <c r="C162" s="11" t="n">
-        <v>55.9482</v>
+        <v>69.99460000000001</v>
       </c>
       <c r="D162" s="11" t="n">
-        <v>39.775</v>
+        <v>53.4524</v>
       </c>
       <c r="E162" s="11" t="n">
-        <v>12.0653</v>
+        <v>17.6309</v>
       </c>
       <c r="F162" s="11" t="n">
-        <v>87.93470000000001</v>
+        <v>82.3691</v>
       </c>
       <c r="G162" s="11" t="n">
-        <v>-0.2174</v>
+        <v>-1.3377</v>
       </c>
       <c r="H162" s="11" t="n">
-        <v>51.9192</v>
+        <v>46.371</v>
       </c>
       <c r="I162" s="11" t="n">
-        <v>0.488</v>
+        <v>0.4537</v>
       </c>
       <c r="J162" s="11" t="n">
-        <v>0.7043</v>
+        <v>0.9196</v>
       </c>
       <c r="K162" s="11" t="n">
-        <v>0.5765</v>
+        <v>0.6077</v>
       </c>
     </row>
     <row r="163">
@@ -6975,31 +6975,31 @@
         </is>
       </c>
       <c r="C164" s="3" t="n">
-        <v>182.3688</v>
+        <v>153.9708</v>
       </c>
       <c r="D164" s="3" t="n">
-        <v>142.8367</v>
+        <v>132.4523</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>12.4396</v>
+        <v>10.9582</v>
       </c>
       <c r="F164" s="3" t="n">
-        <v>87.5604</v>
+        <v>89.04179999999999</v>
       </c>
       <c r="G164" s="3" t="n">
-        <v>-1.2981</v>
+        <v>-2.7146</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>50.9091</v>
+        <v>50.8065</v>
       </c>
       <c r="I164" s="3" t="n">
-        <v>0.5846</v>
+        <v>0.7222</v>
       </c>
       <c r="J164" s="3" t="n">
-        <v>0.1496</v>
+        <v>0.1</v>
       </c>
       <c r="K164" s="3" t="n">
-        <v>0.2382</v>
+        <v>0.1757</v>
       </c>
     </row>
     <row r="165">
@@ -7131,31 +7131,31 @@
         </is>
       </c>
       <c r="C168" s="11" t="n">
-        <v>182.0059</v>
+        <v>154.1266</v>
       </c>
       <c r="D168" s="11" t="n">
-        <v>142.4776</v>
+        <v>132.599</v>
       </c>
       <c r="E168" s="11" t="n">
-        <v>12.4073</v>
+        <v>10.9704</v>
       </c>
       <c r="F168" s="11" t="n">
-        <v>87.59269999999999</v>
+        <v>89.0296</v>
       </c>
       <c r="G168" s="11" t="n">
-        <v>-1.289</v>
+        <v>-2.7222</v>
       </c>
       <c r="H168" s="11" t="n">
-        <v>50.7071</v>
+        <v>50</v>
       </c>
       <c r="I168" s="11" t="n">
-        <v>0.5758</v>
+        <v>0.6667</v>
       </c>
       <c r="J168" s="11" t="n">
-        <v>0.1496</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="K168" s="11" t="n">
-        <v>0.2375</v>
+        <v>0.1622</v>
       </c>
     </row>
     <row r="169">
@@ -7209,31 +7209,31 @@
         </is>
       </c>
       <c r="C170" s="3" t="n">
-        <v>39.0371</v>
+        <v>31.6897</v>
       </c>
       <c r="D170" s="3" t="n">
-        <v>32.2971</v>
+        <v>24.7859</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>7.8557</v>
+        <v>6.3822</v>
       </c>
       <c r="F170" s="3" t="n">
-        <v>92.1443</v>
+        <v>93.6178</v>
       </c>
       <c r="G170" s="3" t="n">
-        <v>-0.7435</v>
+        <v>-0.9936</v>
       </c>
       <c r="H170" s="3" t="n">
-        <v>51.9192</v>
+        <v>52.8226</v>
       </c>
       <c r="I170" s="3" t="n">
-        <v>0.5078</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="J170" s="3" t="n">
-        <v>0.2708</v>
+        <v>0.839</v>
       </c>
       <c r="K170" s="3" t="n">
-        <v>0.3533</v>
+        <v>0.6286</v>
       </c>
     </row>
     <row r="171">
@@ -7365,31 +7365,31 @@
         </is>
       </c>
       <c r="C174" s="11" t="n">
-        <v>38.9358</v>
+        <v>31.9895</v>
       </c>
       <c r="D174" s="11" t="n">
-        <v>32.2145</v>
+        <v>25.0336</v>
       </c>
       <c r="E174" s="11" t="n">
-        <v>7.8366</v>
+        <v>6.4464</v>
       </c>
       <c r="F174" s="11" t="n">
-        <v>92.1634</v>
+        <v>93.5536</v>
       </c>
       <c r="G174" s="11" t="n">
-        <v>-0.7345</v>
+        <v>-1.0315</v>
       </c>
       <c r="H174" s="11" t="n">
-        <v>52.1212</v>
+        <v>52.8226</v>
       </c>
       <c r="I174" s="11" t="n">
-        <v>0.5118</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="J174" s="11" t="n">
-        <v>0.2708</v>
+        <v>0.8559</v>
       </c>
       <c r="K174" s="11" t="n">
-        <v>0.3542</v>
+        <v>0.6332</v>
       </c>
     </row>
     <row r="175">
@@ -7443,31 +7443,31 @@
         </is>
       </c>
       <c r="C176" s="3" t="n">
-        <v>287.2986</v>
+        <v>378.914</v>
       </c>
       <c r="D176" s="3" t="n">
-        <v>224.4529</v>
+        <v>319.5361</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>6.036</v>
+        <v>8.022500000000001</v>
       </c>
       <c r="F176" s="3" t="n">
-        <v>93.964</v>
+        <v>91.97750000000001</v>
       </c>
       <c r="G176" s="3" t="n">
-        <v>-0.0541</v>
+        <v>-1.6269</v>
       </c>
       <c r="H176" s="3" t="n">
-        <v>51.3131</v>
+        <v>52.0161</v>
       </c>
       <c r="I176" s="3" t="n">
-        <v>0.4938</v>
+        <v>0.5588</v>
       </c>
       <c r="J176" s="3" t="n">
-        <v>0.5</v>
+        <v>0.1545</v>
       </c>
       <c r="K176" s="3" t="n">
-        <v>0.4969</v>
+        <v>0.242</v>
       </c>
     </row>
     <row r="177">
@@ -7599,31 +7599,31 @@
         </is>
       </c>
       <c r="C180" s="11" t="n">
-        <v>287.794</v>
+        <v>373.9908</v>
       </c>
       <c r="D180" s="11" t="n">
-        <v>224.5507</v>
+        <v>314.854</v>
       </c>
       <c r="E180" s="11" t="n">
-        <v>6.0351</v>
+        <v>7.9046</v>
       </c>
       <c r="F180" s="11" t="n">
-        <v>93.9649</v>
+        <v>92.0954</v>
       </c>
       <c r="G180" s="11" t="n">
-        <v>-0.0578</v>
+        <v>-1.559</v>
       </c>
       <c r="H180" s="11" t="n">
-        <v>51.5152</v>
+        <v>52.4194</v>
       </c>
       <c r="I180" s="11" t="n">
-        <v>0.4958</v>
+        <v>0.5714</v>
       </c>
       <c r="J180" s="11" t="n">
-        <v>0.5</v>
+        <v>0.1626</v>
       </c>
       <c r="K180" s="11" t="n">
-        <v>0.4979</v>
+        <v>0.2532</v>
       </c>
     </row>
     <row r="181">
@@ -7677,31 +7677,31 @@
         </is>
       </c>
       <c r="C182" s="3" t="n">
-        <v>714.7909</v>
+        <v>792.8978</v>
       </c>
       <c r="D182" s="3" t="n">
-        <v>596.9787</v>
+        <v>658.322</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>12.1716</v>
+        <v>14.3912</v>
       </c>
       <c r="F182" s="3" t="n">
-        <v>87.8284</v>
+        <v>85.6088</v>
       </c>
       <c r="G182" s="3" t="n">
-        <v>-0.0004</v>
+        <v>-0.1156</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>50.101</v>
+        <v>51.2097</v>
       </c>
       <c r="I182" s="3" t="n">
-        <v>0.5022</v>
+        <v>0.4968</v>
       </c>
       <c r="J182" s="3" t="n">
-        <v>0.4556</v>
+        <v>0.65</v>
       </c>
       <c r="K182" s="3" t="n">
-        <v>0.4778</v>
+        <v>0.5632</v>
       </c>
     </row>
     <row r="183">
@@ -7833,31 +7833,31 @@
         </is>
       </c>
       <c r="C186" s="11" t="n">
-        <v>715.5246</v>
+        <v>792.1772</v>
       </c>
       <c r="D186" s="11" t="n">
-        <v>595.5685999999999</v>
+        <v>657.678</v>
       </c>
       <c r="E186" s="11" t="n">
-        <v>12.1928</v>
+        <v>14.3729</v>
       </c>
       <c r="F186" s="11" t="n">
-        <v>87.80719999999999</v>
+        <v>85.6271</v>
       </c>
       <c r="G186" s="11" t="n">
-        <v>-0.0025</v>
+        <v>-0.1135</v>
       </c>
       <c r="H186" s="11" t="n">
-        <v>49.899</v>
+        <v>51.2097</v>
       </c>
       <c r="I186" s="11" t="n">
-        <v>0.5</v>
+        <v>0.4968</v>
       </c>
       <c r="J186" s="11" t="n">
-        <v>0.4758</v>
+        <v>0.65</v>
       </c>
       <c r="K186" s="11" t="n">
-        <v>0.4876</v>
+        <v>0.5632</v>
       </c>
     </row>
     <row r="187">
@@ -7911,31 +7911,31 @@
         </is>
       </c>
       <c r="C188" s="3" t="n">
-        <v>388.4212</v>
+        <v>318.3166</v>
       </c>
       <c r="D188" s="3" t="n">
-        <v>306.4257</v>
+        <v>256.0688</v>
       </c>
       <c r="E188" s="3" t="n">
-        <v>9.3611</v>
+        <v>7.3396</v>
       </c>
       <c r="F188" s="3" t="n">
-        <v>90.63890000000001</v>
+        <v>92.6604</v>
       </c>
       <c r="G188" s="3" t="n">
-        <v>-0.5028</v>
+        <v>-0.7621</v>
       </c>
       <c r="H188" s="3" t="n">
-        <v>52.3232</v>
+        <v>56.4516</v>
       </c>
       <c r="I188" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5938</v>
       </c>
       <c r="J188" s="3" t="n">
-        <v>0.2789</v>
+        <v>0.3167</v>
       </c>
       <c r="K188" s="3" t="n">
-        <v>0.3723</v>
+        <v>0.413</v>
       </c>
     </row>
     <row r="189">
@@ -8067,31 +8067,31 @@
         </is>
       </c>
       <c r="C192" s="11" t="n">
-        <v>390.7641</v>
+        <v>321.8854</v>
       </c>
       <c r="D192" s="11" t="n">
-        <v>308.4356</v>
+        <v>258.725</v>
       </c>
       <c r="E192" s="11" t="n">
-        <v>9.417899999999999</v>
+        <v>7.4118</v>
       </c>
       <c r="F192" s="11" t="n">
-        <v>90.5821</v>
+        <v>92.5882</v>
       </c>
       <c r="G192" s="11" t="n">
-        <v>-0.521</v>
+        <v>-0.8018999999999999</v>
       </c>
       <c r="H192" s="11" t="n">
-        <v>52.3232</v>
+        <v>56.4516</v>
       </c>
       <c r="I192" s="11" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.5968</v>
       </c>
       <c r="J192" s="11" t="n">
-        <v>0.2749</v>
+        <v>0.3083</v>
       </c>
       <c r="K192" s="11" t="n">
-        <v>0.369</v>
+        <v>0.4066</v>
       </c>
     </row>
     <row r="193">
@@ -8145,31 +8145,31 @@
         </is>
       </c>
       <c r="C194" s="3" t="n">
-        <v>1855.2544</v>
+        <v>2599.8532</v>
       </c>
       <c r="D194" s="3" t="n">
-        <v>1342.4917</v>
+        <v>2154.2414</v>
       </c>
       <c r="E194" s="3" t="n">
-        <v>9.4047</v>
+        <v>13.9557</v>
       </c>
       <c r="F194" s="3" t="n">
-        <v>90.59529999999999</v>
+        <v>86.04430000000001</v>
       </c>
       <c r="G194" s="3" t="n">
-        <v>-0.1779</v>
+        <v>-2.1446</v>
       </c>
       <c r="H194" s="3" t="n">
-        <v>50.101</v>
+        <v>51.2097</v>
       </c>
       <c r="I194" s="3" t="n">
-        <v>0.4936</v>
+        <v>0.7692</v>
       </c>
       <c r="J194" s="3" t="n">
-        <v>0.4713</v>
+        <v>0.0781</v>
       </c>
       <c r="K194" s="3" t="n">
-        <v>0.4822</v>
+        <v>0.1418</v>
       </c>
     </row>
     <row r="195">
@@ -8301,31 +8301,31 @@
         </is>
       </c>
       <c r="C198" s="11" t="n">
-        <v>1840.6624</v>
+        <v>2599.4524</v>
       </c>
       <c r="D198" s="11" t="n">
-        <v>1340.7212</v>
+        <v>2153.8027</v>
       </c>
       <c r="E198" s="11" t="n">
-        <v>9.4194</v>
+        <v>13.9527</v>
       </c>
       <c r="F198" s="11" t="n">
-        <v>90.5806</v>
+        <v>86.04730000000001</v>
       </c>
       <c r="G198" s="11" t="n">
-        <v>-0.1594</v>
+        <v>-2.1436</v>
       </c>
       <c r="H198" s="11" t="n">
-        <v>50.9091</v>
+        <v>51.2097</v>
       </c>
       <c r="I198" s="11" t="n">
-        <v>0.5021</v>
+        <v>0.7692</v>
       </c>
       <c r="J198" s="11" t="n">
-        <v>0.4959</v>
+        <v>0.0781</v>
       </c>
       <c r="K198" s="11" t="n">
-        <v>0.499</v>
+        <v>0.1418</v>
       </c>
     </row>
     <row r="199">
@@ -8379,31 +8379,31 @@
         </is>
       </c>
       <c r="C200" s="3" t="n">
-        <v>125.6931</v>
+        <v>119.1098</v>
       </c>
       <c r="D200" s="3" t="n">
-        <v>107.032</v>
+        <v>90.4913</v>
       </c>
       <c r="E200" s="3" t="n">
-        <v>9.1143</v>
+        <v>6.7818</v>
       </c>
       <c r="F200" s="3" t="n">
-        <v>90.8857</v>
+        <v>93.2182</v>
       </c>
       <c r="G200" s="3" t="n">
-        <v>-0.5455</v>
+        <v>-0.4902</v>
       </c>
       <c r="H200" s="3" t="n">
-        <v>52.3232</v>
+        <v>55.2419</v>
       </c>
       <c r="I200" s="3" t="n">
-        <v>0.5112</v>
+        <v>0.6061</v>
       </c>
       <c r="J200" s="3" t="n">
-        <v>0.8367</v>
+        <v>0.32</v>
       </c>
       <c r="K200" s="3" t="n">
-        <v>0.6347</v>
+        <v>0.4188</v>
       </c>
     </row>
     <row r="201">
@@ -8535,31 +8535,31 @@
         </is>
       </c>
       <c r="C204" s="11" t="n">
-        <v>122.5456</v>
+        <v>119.4569</v>
       </c>
       <c r="D204" s="11" t="n">
-        <v>103.7511</v>
+        <v>90.77330000000001</v>
       </c>
       <c r="E204" s="11" t="n">
-        <v>8.8222</v>
+        <v>6.8019</v>
       </c>
       <c r="F204" s="11" t="n">
-        <v>91.1778</v>
+        <v>93.1981</v>
       </c>
       <c r="G204" s="11" t="n">
-        <v>-0.4691</v>
+        <v>-0.4989</v>
       </c>
       <c r="H204" s="11" t="n">
-        <v>52.9293</v>
+        <v>55.2419</v>
       </c>
       <c r="I204" s="11" t="n">
-        <v>0.5152</v>
+        <v>0.6061</v>
       </c>
       <c r="J204" s="11" t="n">
-        <v>0.8327</v>
+        <v>0.32</v>
       </c>
       <c r="K204" s="11" t="n">
-        <v>0.6365</v>
+        <v>0.4188</v>
       </c>
     </row>
     <row r="205">
@@ -8613,31 +8613,31 @@
         </is>
       </c>
       <c r="C206" s="3" t="n">
-        <v>31.6717</v>
+        <v>33.727</v>
       </c>
       <c r="D206" s="3" t="n">
-        <v>28.0545</v>
+        <v>24.3625</v>
       </c>
       <c r="E206" s="3" t="n">
-        <v>8.139799999999999</v>
+        <v>6.532</v>
       </c>
       <c r="F206" s="3" t="n">
-        <v>91.86020000000001</v>
+        <v>93.468</v>
       </c>
       <c r="G206" s="3" t="n">
-        <v>-0.0842</v>
+        <v>-0.6635</v>
       </c>
       <c r="H206" s="3" t="n">
-        <v>51.7172</v>
+        <v>55.6452</v>
       </c>
       <c r="I206" s="3" t="n">
-        <v>0.5031</v>
+        <v>0.5797</v>
       </c>
       <c r="J206" s="3" t="n">
-        <v>0.6639</v>
+        <v>0.3306</v>
       </c>
       <c r="K206" s="3" t="n">
-        <v>0.5725</v>
+        <v>0.4211</v>
       </c>
     </row>
     <row r="207">
@@ -8769,31 +8769,31 @@
         </is>
       </c>
       <c r="C210" s="11" t="n">
-        <v>31.834</v>
+        <v>33.3385</v>
       </c>
       <c r="D210" s="11" t="n">
-        <v>28.222</v>
+        <v>24.1029</v>
       </c>
       <c r="E210" s="11" t="n">
-        <v>8.1991</v>
+        <v>6.4653</v>
       </c>
       <c r="F210" s="11" t="n">
-        <v>91.8009</v>
+        <v>93.5347</v>
       </c>
       <c r="G210" s="11" t="n">
-        <v>-0.0953</v>
+        <v>-0.6254</v>
       </c>
       <c r="H210" s="11" t="n">
-        <v>52.5253</v>
+        <v>55.6452</v>
       </c>
       <c r="I210" s="11" t="n">
-        <v>0.5093</v>
+        <v>0.5775</v>
       </c>
       <c r="J210" s="11" t="n">
-        <v>0.6805</v>
+        <v>0.3388</v>
       </c>
       <c r="K210" s="11" t="n">
-        <v>0.5826</v>
+        <v>0.4271</v>
       </c>
     </row>
     <row r="211">
@@ -8847,31 +8847,31 @@
         </is>
       </c>
       <c r="C212" s="3" t="n">
-        <v>30.9605</v>
+        <v>30.5774</v>
       </c>
       <c r="D212" s="3" t="n">
-        <v>27.9979</v>
+        <v>21.6333</v>
       </c>
       <c r="E212" s="3" t="n">
-        <v>11.7433</v>
+        <v>7.9971</v>
       </c>
       <c r="F212" s="3" t="n">
-        <v>88.2567</v>
+        <v>92.0029</v>
       </c>
       <c r="G212" s="3" t="n">
-        <v>-0.635</v>
+        <v>-0.7193000000000001</v>
       </c>
       <c r="H212" s="3" t="n">
-        <v>50.9091</v>
+        <v>53.2258</v>
       </c>
       <c r="I212" s="3" t="n">
-        <v>0.496</v>
+        <v>0.5593</v>
       </c>
       <c r="J212" s="3" t="n">
-        <v>0.7792</v>
+        <v>0.2683</v>
       </c>
       <c r="K212" s="3" t="n">
-        <v>0.6062</v>
+        <v>0.3626</v>
       </c>
     </row>
     <row r="213">
@@ -9003,31 +9003,31 @@
         </is>
       </c>
       <c r="C216" s="11" t="n">
-        <v>32.9141</v>
+        <v>30.8375</v>
       </c>
       <c r="D216" s="11" t="n">
-        <v>29.6888</v>
+        <v>21.8509</v>
       </c>
       <c r="E216" s="11" t="n">
-        <v>12.5073</v>
+        <v>8.077999999999999</v>
       </c>
       <c r="F216" s="11" t="n">
-        <v>87.4927</v>
+        <v>91.922</v>
       </c>
       <c r="G216" s="11" t="n">
-        <v>-0.8478</v>
+        <v>-0.7487</v>
       </c>
       <c r="H216" s="11" t="n">
-        <v>50.7071</v>
+        <v>52.8226</v>
       </c>
       <c r="I216" s="11" t="n">
-        <v>0.4949</v>
+        <v>0.5556</v>
       </c>
       <c r="J216" s="11" t="n">
-        <v>0.8083</v>
+        <v>0.2439</v>
       </c>
       <c r="K216" s="11" t="n">
-        <v>0.6139</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="217">
@@ -9081,31 +9081,31 @@
         </is>
       </c>
       <c r="C218" s="3" t="n">
-        <v>35.9584</v>
+        <v>16.7877</v>
       </c>
       <c r="D218" s="3" t="n">
-        <v>30.5128</v>
+        <v>13.4493</v>
       </c>
       <c r="E218" s="3" t="n">
-        <v>11.0314</v>
+        <v>4.8047</v>
       </c>
       <c r="F218" s="3" t="n">
-        <v>88.9686</v>
+        <v>95.1953</v>
       </c>
       <c r="G218" s="3" t="n">
-        <v>-2.1249</v>
+        <v>-0.0304</v>
       </c>
       <c r="H218" s="3" t="n">
-        <v>51.3131</v>
+        <v>53.2258</v>
       </c>
       <c r="I218" s="3" t="n">
-        <v>0.5011</v>
+        <v>0.531</v>
       </c>
       <c r="J218" s="3" t="n">
-        <v>0.9504</v>
+        <v>0.616</v>
       </c>
       <c r="K218" s="3" t="n">
-        <v>0.6562</v>
+        <v>0.5704</v>
       </c>
     </row>
     <row r="219">
@@ -9237,31 +9237,31 @@
         </is>
       </c>
       <c r="C222" s="11" t="n">
-        <v>35.8169</v>
+        <v>16.9533</v>
       </c>
       <c r="D222" s="11" t="n">
-        <v>30.368</v>
+        <v>13.6218</v>
       </c>
       <c r="E222" s="11" t="n">
-        <v>10.9802</v>
+        <v>4.879</v>
       </c>
       <c r="F222" s="11" t="n">
-        <v>89.0198</v>
+        <v>95.121</v>
       </c>
       <c r="G222" s="11" t="n">
-        <v>-2.1003</v>
+        <v>-0.0508</v>
       </c>
       <c r="H222" s="11" t="n">
-        <v>50.9091</v>
+        <v>54.0323</v>
       </c>
       <c r="I222" s="11" t="n">
-        <v>0.4989</v>
+        <v>0.5369</v>
       </c>
       <c r="J222" s="11" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.64</v>
       </c>
       <c r="K222" s="11" t="n">
-        <v>0.6514</v>
+        <v>0.5839</v>
       </c>
     </row>
     <row r="223">
@@ -9315,31 +9315,31 @@
         </is>
       </c>
       <c r="C224" s="3" t="n">
-        <v>215.499</v>
+        <v>138.13</v>
       </c>
       <c r="D224" s="3" t="n">
-        <v>191.1815</v>
+        <v>121.1607</v>
       </c>
       <c r="E224" s="3" t="n">
-        <v>14.475</v>
+        <v>8.8573</v>
       </c>
       <c r="F224" s="3" t="n">
-        <v>85.52500000000001</v>
+        <v>91.1427</v>
       </c>
       <c r="G224" s="3" t="n">
-        <v>-3.672</v>
+        <v>-2.3648</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>49.4949</v>
+        <v>48.3871</v>
       </c>
       <c r="I224" s="3" t="n">
-        <v>0.4918</v>
+        <v>0.4722</v>
       </c>
       <c r="J224" s="3" t="n">
-        <v>0.9959</v>
+        <v>0.8793</v>
       </c>
       <c r="K224" s="3" t="n">
-        <v>0.6585</v>
+        <v>0.6145</v>
       </c>
     </row>
     <row r="225">
@@ -9471,31 +9471,31 @@
         </is>
       </c>
       <c r="C228" s="11" t="n">
-        <v>219.2949</v>
+        <v>138.1131</v>
       </c>
       <c r="D228" s="11" t="n">
-        <v>195.3913</v>
+        <v>121.1567</v>
       </c>
       <c r="E228" s="11" t="n">
-        <v>14.7826</v>
+        <v>8.8569</v>
       </c>
       <c r="F228" s="11" t="n">
-        <v>85.2174</v>
+        <v>91.1431</v>
       </c>
       <c r="G228" s="11" t="n">
-        <v>-3.838</v>
+        <v>-2.364</v>
       </c>
       <c r="H228" s="11" t="n">
-        <v>49.0909</v>
+        <v>48.3871</v>
       </c>
       <c r="I228" s="11" t="n">
-        <v>0.4898</v>
+        <v>0.4722</v>
       </c>
       <c r="J228" s="11" t="n">
-        <v>0.9959</v>
+        <v>0.8793</v>
       </c>
       <c r="K228" s="11" t="n">
-        <v>0.6567</v>
+        <v>0.6145</v>
       </c>
     </row>
     <row r="229">
@@ -9549,31 +9549,31 @@
         </is>
       </c>
       <c r="C230" s="3" t="n">
-        <v>310.7653</v>
+        <v>137.0765</v>
       </c>
       <c r="D230" s="3" t="n">
-        <v>270.7281</v>
+        <v>102.9647</v>
       </c>
       <c r="E230" s="3" t="n">
-        <v>14.6059</v>
+        <v>5.1963</v>
       </c>
       <c r="F230" s="3" t="n">
-        <v>85.39409999999999</v>
+        <v>94.80370000000001</v>
       </c>
       <c r="G230" s="3" t="n">
-        <v>-1.6427</v>
+        <v>-0.8171</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>49.697</v>
+        <v>52.8226</v>
       </c>
       <c r="I230" s="3" t="n">
-        <v>0.4607</v>
+        <v>0.5926</v>
       </c>
       <c r="J230" s="3" t="n">
-        <v>0.1694</v>
+        <v>0.252</v>
       </c>
       <c r="K230" s="3" t="n">
-        <v>0.2477</v>
+        <v>0.3536</v>
       </c>
     </row>
     <row r="231">
@@ -9705,31 +9705,31 @@
         </is>
       </c>
       <c r="C234" s="11" t="n">
-        <v>312.2496</v>
+        <v>137.9136</v>
       </c>
       <c r="D234" s="11" t="n">
-        <v>271.9271</v>
+        <v>103.7145</v>
       </c>
       <c r="E234" s="11" t="n">
-        <v>14.6668</v>
+        <v>5.2342</v>
       </c>
       <c r="F234" s="11" t="n">
-        <v>85.33320000000001</v>
+        <v>94.7658</v>
       </c>
       <c r="G234" s="11" t="n">
-        <v>-1.668</v>
+        <v>-0.8393</v>
       </c>
       <c r="H234" s="11" t="n">
-        <v>49.697</v>
+        <v>52.4194</v>
       </c>
       <c r="I234" s="11" t="n">
-        <v>0.4598</v>
+        <v>0.5957</v>
       </c>
       <c r="J234" s="11" t="n">
-        <v>0.1653</v>
+        <v>0.2205</v>
       </c>
       <c r="K234" s="11" t="n">
-        <v>0.2432</v>
+        <v>0.3218</v>
       </c>
     </row>
     <row r="235">
@@ -9783,31 +9783,31 @@
         </is>
       </c>
       <c r="C236" s="3" t="n">
-        <v>128.8171</v>
+        <v>197.5735</v>
       </c>
       <c r="D236" s="3" t="n">
-        <v>101.4993</v>
+        <v>165.1347</v>
       </c>
       <c r="E236" s="3" t="n">
-        <v>11.1289</v>
+        <v>16.1583</v>
       </c>
       <c r="F236" s="3" t="n">
-        <v>88.8711</v>
+        <v>83.8417</v>
       </c>
       <c r="G236" s="3" t="n">
-        <v>-0.0592</v>
+        <v>-2.2533</v>
       </c>
       <c r="H236" s="3" t="n">
-        <v>50.303</v>
+        <v>48.7903</v>
       </c>
       <c r="I236" s="3" t="n">
-        <v>0.5122</v>
+        <v>0.6471</v>
       </c>
       <c r="J236" s="3" t="n">
-        <v>0.581</v>
+        <v>0.0833</v>
       </c>
       <c r="K236" s="3" t="n">
-        <v>0.5444</v>
+        <v>0.1477</v>
       </c>
     </row>
     <row r="237">
@@ -9939,31 +9939,31 @@
         </is>
       </c>
       <c r="C240" s="11" t="n">
-        <v>129.4716</v>
+        <v>197.0894</v>
       </c>
       <c r="D240" s="11" t="n">
-        <v>101.1162</v>
+        <v>164.6298</v>
       </c>
       <c r="E240" s="11" t="n">
-        <v>11.0474</v>
+        <v>16.1065</v>
       </c>
       <c r="F240" s="11" t="n">
-        <v>88.9526</v>
+        <v>83.8935</v>
       </c>
       <c r="G240" s="11" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-2.2373</v>
       </c>
       <c r="H240" s="11" t="n">
-        <v>50.9091</v>
+        <v>48.7903</v>
       </c>
       <c r="I240" s="11" t="n">
-        <v>0.5177</v>
+        <v>0.6471</v>
       </c>
       <c r="J240" s="11" t="n">
-        <v>0.5770999999999999</v>
+        <v>0.0833</v>
       </c>
       <c r="K240" s="11" t="n">
-        <v>0.5458</v>
+        <v>0.1477</v>
       </c>
     </row>
     <row r="241">
@@ -10017,31 +10017,31 @@
         </is>
       </c>
       <c r="C242" s="3" t="n">
-        <v>255.3108</v>
+        <v>250.2903</v>
       </c>
       <c r="D242" s="3" t="n">
-        <v>191.6642</v>
+        <v>210.66</v>
       </c>
       <c r="E242" s="3" t="n">
-        <v>22.6102</v>
+        <v>22.484</v>
       </c>
       <c r="F242" s="3" t="n">
-        <v>77.38979999999999</v>
+        <v>77.51600000000001</v>
       </c>
       <c r="G242" s="3" t="n">
-        <v>-1.2383</v>
+        <v>-1.3311</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>49.4949</v>
+        <v>47.5806</v>
       </c>
       <c r="I242" s="3" t="n">
-        <v>0.5357</v>
+        <v>0.5238</v>
       </c>
       <c r="J242" s="3" t="n">
-        <v>0.0595</v>
+        <v>0.2481</v>
       </c>
       <c r="K242" s="3" t="n">
-        <v>0.1071</v>
+        <v>0.3367</v>
       </c>
     </row>
     <row r="243">
@@ -10173,31 +10173,31 @@
         </is>
       </c>
       <c r="C246" s="11" t="n">
-        <v>255.5934</v>
+        <v>251.6138</v>
       </c>
       <c r="D246" s="11" t="n">
-        <v>192.0033</v>
+        <v>211.5809</v>
       </c>
       <c r="E246" s="11" t="n">
-        <v>22.657</v>
+        <v>22.5638</v>
       </c>
       <c r="F246" s="11" t="n">
-        <v>77.343</v>
+        <v>77.4362</v>
       </c>
       <c r="G246" s="11" t="n">
-        <v>-1.2432</v>
+        <v>-1.3558</v>
       </c>
       <c r="H246" s="11" t="n">
-        <v>49.2929</v>
+        <v>48.7903</v>
       </c>
       <c r="I246" s="11" t="n">
-        <v>0.5185</v>
+        <v>0.5517</v>
       </c>
       <c r="J246" s="11" t="n">
-        <v>0.0556</v>
+        <v>0.2406</v>
       </c>
       <c r="K246" s="11" t="n">
-        <v>0.1004</v>
+        <v>0.3351</v>
       </c>
     </row>
     <row r="247">
@@ -10251,31 +10251,31 @@
         </is>
       </c>
       <c r="C248" s="3" t="n">
-        <v>187.1618</v>
+        <v>99.11839999999999</v>
       </c>
       <c r="D248" s="3" t="n">
-        <v>167.5579</v>
+        <v>80.3193</v>
       </c>
       <c r="E248" s="3" t="n">
-        <v>9.5139</v>
+        <v>4.5745</v>
       </c>
       <c r="F248" s="3" t="n">
-        <v>90.48609999999999</v>
+        <v>95.4255</v>
       </c>
       <c r="G248" s="3" t="n">
-        <v>-3.9864</v>
+        <v>-0.3434</v>
       </c>
       <c r="H248" s="3" t="n">
-        <v>48.2828</v>
+        <v>51.2097</v>
       </c>
       <c r="I248" s="3" t="n">
-        <v>1</v>
+        <v>0.6216</v>
       </c>
       <c r="J248" s="3" t="n">
-        <v>0.0266</v>
+        <v>0.3309</v>
       </c>
       <c r="K248" s="3" t="n">
-        <v>0.0519</v>
+        <v>0.4319</v>
       </c>
     </row>
     <row r="249">
@@ -10407,31 +10407,31 @@
         </is>
       </c>
       <c r="C252" s="11" t="n">
-        <v>189.5862</v>
+        <v>99.3103</v>
       </c>
       <c r="D252" s="11" t="n">
-        <v>170.1888</v>
+        <v>80.4808</v>
       </c>
       <c r="E252" s="11" t="n">
-        <v>9.666499999999999</v>
+        <v>4.5832</v>
       </c>
       <c r="F252" s="11" t="n">
-        <v>90.3335</v>
+        <v>95.41679999999999</v>
       </c>
       <c r="G252" s="11" t="n">
-        <v>-4.1164</v>
+        <v>-0.3486</v>
       </c>
       <c r="H252" s="11" t="n">
-        <v>48.2828</v>
+        <v>51.2097</v>
       </c>
       <c r="I252" s="11" t="n">
-        <v>1</v>
+        <v>0.6216</v>
       </c>
       <c r="J252" s="11" t="n">
-        <v>0.0266</v>
+        <v>0.3309</v>
       </c>
       <c r="K252" s="11" t="n">
-        <v>0.0519</v>
+        <v>0.4319</v>
       </c>
     </row>
     <row r="253">
@@ -10485,31 +10485,31 @@
         </is>
       </c>
       <c r="C254" s="3" t="n">
-        <v>93.4675</v>
+        <v>57.0531</v>
       </c>
       <c r="D254" s="3" t="n">
-        <v>69.2778</v>
+        <v>48.0164</v>
       </c>
       <c r="E254" s="3" t="n">
-        <v>6.8315</v>
+        <v>4.2006</v>
       </c>
       <c r="F254" s="3" t="n">
-        <v>93.16849999999999</v>
+        <v>95.79940000000001</v>
       </c>
       <c r="G254" s="3" t="n">
-        <v>-0.2021</v>
+        <v>-0.4421</v>
       </c>
       <c r="H254" s="3" t="n">
-        <v>55.9596</v>
+        <v>56.0484</v>
       </c>
       <c r="I254" s="3" t="n">
-        <v>0.543</v>
+        <v>0.5735</v>
       </c>
       <c r="J254" s="3" t="n">
-        <v>0.6502</v>
+        <v>0.3277</v>
       </c>
       <c r="K254" s="3" t="n">
-        <v>0.5918</v>
+        <v>0.4171</v>
       </c>
     </row>
     <row r="255">
@@ -10641,31 +10641,31 @@
         </is>
       </c>
       <c r="C258" s="11" t="n">
-        <v>92.53100000000001</v>
+        <v>57.2434</v>
       </c>
       <c r="D258" s="11" t="n">
-        <v>68.87</v>
+        <v>48.1743</v>
       </c>
       <c r="E258" s="11" t="n">
-        <v>6.7811</v>
+        <v>4.2138</v>
       </c>
       <c r="F258" s="11" t="n">
-        <v>93.2189</v>
+        <v>95.78619999999999</v>
       </c>
       <c r="G258" s="11" t="n">
-        <v>-0.1781</v>
+        <v>-0.4517</v>
       </c>
       <c r="H258" s="11" t="n">
-        <v>56.5657</v>
+        <v>56.0484</v>
       </c>
       <c r="I258" s="11" t="n">
-        <v>0.5486</v>
+        <v>0.5735</v>
       </c>
       <c r="J258" s="11" t="n">
-        <v>0.6502</v>
+        <v>0.3277</v>
       </c>
       <c r="K258" s="11" t="n">
-        <v>0.5951</v>
+        <v>0.4171</v>
       </c>
     </row>
     <row r="259">
@@ -10719,31 +10719,31 @@
         </is>
       </c>
       <c r="C260" s="3" t="n">
-        <v>24.5549</v>
+        <v>28.76</v>
       </c>
       <c r="D260" s="3" t="n">
-        <v>20.687</v>
+        <v>23.0238</v>
       </c>
       <c r="E260" s="3" t="n">
-        <v>13.0419</v>
+        <v>11.8932</v>
       </c>
       <c r="F260" s="3" t="n">
-        <v>86.9581</v>
+        <v>88.10680000000001</v>
       </c>
       <c r="G260" s="3" t="n">
-        <v>-0.0129</v>
+        <v>-1.4324</v>
       </c>
       <c r="H260" s="3" t="n">
-        <v>50.9091</v>
+        <v>50.8065</v>
       </c>
       <c r="I260" s="3" t="n">
-        <v>0.5132</v>
+        <v>0.5833</v>
       </c>
       <c r="J260" s="3" t="n">
-        <v>0.6215000000000001</v>
+        <v>0.1641</v>
       </c>
       <c r="K260" s="3" t="n">
-        <v>0.5622</v>
+        <v>0.2561</v>
       </c>
     </row>
     <row r="261">
@@ -10875,31 +10875,31 @@
         </is>
       </c>
       <c r="C264" s="11" t="n">
-        <v>24.5378</v>
+        <v>28.4788</v>
       </c>
       <c r="D264" s="11" t="n">
-        <v>20.6526</v>
+        <v>22.7631</v>
       </c>
       <c r="E264" s="11" t="n">
-        <v>13.0084</v>
+        <v>11.7567</v>
       </c>
       <c r="F264" s="11" t="n">
-        <v>86.99160000000001</v>
+        <v>88.2433</v>
       </c>
       <c r="G264" s="11" t="n">
-        <v>-0.0115</v>
+        <v>-1.3851</v>
       </c>
       <c r="H264" s="11" t="n">
-        <v>50.9091</v>
+        <v>50.8065</v>
       </c>
       <c r="I264" s="11" t="n">
-        <v>0.5132</v>
+        <v>0.5789</v>
       </c>
       <c r="J264" s="11" t="n">
-        <v>0.6175</v>
+        <v>0.1719</v>
       </c>
       <c r="K264" s="11" t="n">
-        <v>0.5606</v>
+        <v>0.2651</v>
       </c>
     </row>
     <row r="265">
@@ -10953,31 +10953,31 @@
         </is>
       </c>
       <c r="C266" s="3" t="n">
-        <v>757.362</v>
+        <v>628.0782</v>
       </c>
       <c r="D266" s="3" t="n">
-        <v>629.5311</v>
+        <v>521.9027</v>
       </c>
       <c r="E266" s="3" t="n">
-        <v>22.6549</v>
+        <v>21.0058</v>
       </c>
       <c r="F266" s="3" t="n">
-        <v>77.3451</v>
+        <v>78.99420000000001</v>
       </c>
       <c r="G266" s="3" t="n">
-        <v>-0.632</v>
+        <v>-2.2309</v>
       </c>
       <c r="H266" s="3" t="n">
-        <v>47.0707</v>
+        <v>43.1452</v>
       </c>
       <c r="I266" s="3" t="n">
-        <v>0.4419</v>
+        <v>0.4315</v>
       </c>
       <c r="J266" s="3" t="n">
-        <v>0.6847</v>
+        <v>1</v>
       </c>
       <c r="K266" s="3" t="n">
-        <v>0.5371</v>
+        <v>0.6028</v>
       </c>
     </row>
     <row r="267">
@@ -11109,31 +11109,31 @@
         </is>
       </c>
       <c r="C270" s="11" t="n">
-        <v>746.4625</v>
+        <v>627.1532999999999</v>
       </c>
       <c r="D270" s="11" t="n">
-        <v>622.2787</v>
+        <v>520.7954999999999</v>
       </c>
       <c r="E270" s="11" t="n">
-        <v>22.3558</v>
+        <v>20.965</v>
       </c>
       <c r="F270" s="11" t="n">
-        <v>77.6442</v>
+        <v>79.035</v>
       </c>
       <c r="G270" s="11" t="n">
-        <v>-0.5853</v>
+        <v>-2.2214</v>
       </c>
       <c r="H270" s="11" t="n">
-        <v>47.0707</v>
+        <v>43.5484</v>
       </c>
       <c r="I270" s="11" t="n">
-        <v>0.4415</v>
+        <v>0.4332</v>
       </c>
       <c r="J270" s="11" t="n">
-        <v>0.6802</v>
+        <v>1</v>
       </c>
       <c r="K270" s="11" t="n">
-        <v>0.5355</v>
+        <v>0.6045</v>
       </c>
     </row>
     <row r="271">
@@ -11187,31 +11187,31 @@
         </is>
       </c>
       <c r="C272" s="3" t="n">
-        <v>167.3125</v>
+        <v>145.9935</v>
       </c>
       <c r="D272" s="3" t="n">
-        <v>140.0458</v>
+        <v>129.3296</v>
       </c>
       <c r="E272" s="3" t="n">
-        <v>9.0961</v>
+        <v>9.190300000000001</v>
       </c>
       <c r="F272" s="3" t="n">
-        <v>90.90389999999999</v>
+        <v>90.80970000000001</v>
       </c>
       <c r="G272" s="3" t="n">
-        <v>-1.6538</v>
+        <v>-1.7497</v>
       </c>
       <c r="H272" s="3" t="n">
-        <v>52.7273</v>
+        <v>50</v>
       </c>
       <c r="I272" s="3" t="n">
-        <v>0.6</v>
+        <v>0.4954</v>
       </c>
       <c r="J272" s="3" t="n">
-        <v>0.1111</v>
+        <v>0.8852</v>
       </c>
       <c r="K272" s="3" t="n">
-        <v>0.1875</v>
+        <v>0.6353</v>
       </c>
     </row>
     <row r="273">
@@ -11343,31 +11343,31 @@
         </is>
       </c>
       <c r="C276" s="11" t="n">
-        <v>164.799</v>
+        <v>144.8432</v>
       </c>
       <c r="D276" s="11" t="n">
-        <v>137.4696</v>
+        <v>128.2587</v>
       </c>
       <c r="E276" s="11" t="n">
-        <v>8.9268</v>
+        <v>9.1134</v>
       </c>
       <c r="F276" s="11" t="n">
-        <v>91.0732</v>
+        <v>90.8866</v>
       </c>
       <c r="G276" s="11" t="n">
-        <v>-1.5747</v>
+        <v>-1.7065</v>
       </c>
       <c r="H276" s="11" t="n">
-        <v>53.1313</v>
+        <v>50</v>
       </c>
       <c r="I276" s="11" t="n">
-        <v>0.6122</v>
+        <v>0.4954</v>
       </c>
       <c r="J276" s="11" t="n">
-        <v>0.1235</v>
+        <v>0.8852</v>
       </c>
       <c r="K276" s="11" t="n">
-        <v>0.2055</v>
+        <v>0.6353</v>
       </c>
     </row>
     <row r="277">
@@ -11421,31 +11421,31 @@
         </is>
       </c>
       <c r="C278" s="3" t="n">
-        <v>600.8171</v>
+        <v>441.6555</v>
       </c>
       <c r="D278" s="3" t="n">
-        <v>475.3632</v>
+        <v>374.6618</v>
       </c>
       <c r="E278" s="3" t="n">
-        <v>12.1089</v>
+        <v>9.146699999999999</v>
       </c>
       <c r="F278" s="3" t="n">
-        <v>87.89109999999999</v>
+        <v>90.8533</v>
       </c>
       <c r="G278" s="3" t="n">
-        <v>-1.3881</v>
+        <v>-0.7071</v>
       </c>
       <c r="H278" s="3" t="n">
-        <v>50.101</v>
+        <v>50.4032</v>
       </c>
       <c r="I278" s="3" t="n">
-        <v>0.5116000000000001</v>
+        <v>0.4848</v>
       </c>
       <c r="J278" s="3" t="n">
-        <v>0.0887</v>
+        <v>0.2645</v>
       </c>
       <c r="K278" s="3" t="n">
-        <v>0.1512</v>
+        <v>0.3422</v>
       </c>
     </row>
     <row r="279">
@@ -11577,31 +11577,31 @@
         </is>
       </c>
       <c r="C282" s="11" t="n">
-        <v>601.9176</v>
+        <v>442.5049</v>
       </c>
       <c r="D282" s="11" t="n">
-        <v>476.5423</v>
+        <v>375.2941</v>
       </c>
       <c r="E282" s="11" t="n">
-        <v>12.1402</v>
+        <v>9.1608</v>
       </c>
       <c r="F282" s="11" t="n">
-        <v>87.85980000000001</v>
+        <v>90.83920000000001</v>
       </c>
       <c r="G282" s="11" t="n">
-        <v>-1.3968</v>
+        <v>-0.7137</v>
       </c>
       <c r="H282" s="11" t="n">
-        <v>50.101</v>
+        <v>50.4032</v>
       </c>
       <c r="I282" s="11" t="n">
-        <v>0.5116000000000001</v>
+        <v>0.4848</v>
       </c>
       <c r="J282" s="11" t="n">
-        <v>0.0887</v>
+        <v>0.2645</v>
       </c>
       <c r="K282" s="11" t="n">
-        <v>0.1512</v>
+        <v>0.3422</v>
       </c>
     </row>
     <row r="283">
@@ -11655,31 +11655,31 @@
         </is>
       </c>
       <c r="C284" s="3" t="n">
-        <v>443.0668</v>
+        <v>277.8357</v>
       </c>
       <c r="D284" s="3" t="n">
-        <v>388.9516</v>
+        <v>240.757</v>
       </c>
       <c r="E284" s="3" t="n">
-        <v>87.9318</v>
+        <v>67.2269</v>
       </c>
       <c r="F284" s="3" t="n">
-        <v>12.0682</v>
+        <v>32.7731</v>
       </c>
       <c r="G284" s="3" t="n">
-        <v>-2.7994</v>
+        <v>-2.7138</v>
       </c>
       <c r="H284" s="3" t="n">
-        <v>47.6768</v>
+        <v>50</v>
       </c>
       <c r="I284" s="3" t="n">
-        <v>0.4641</v>
+        <v>0.4706</v>
       </c>
       <c r="J284" s="3" t="n">
-        <v>0.9425</v>
+        <v>0.9369</v>
       </c>
       <c r="K284" s="3" t="n">
-        <v>0.6219</v>
+        <v>0.6264999999999999</v>
       </c>
     </row>
     <row r="285">
@@ -11811,31 +11811,31 @@
         </is>
       </c>
       <c r="C288" s="11" t="n">
-        <v>443.8825</v>
+        <v>279.0715</v>
       </c>
       <c r="D288" s="11" t="n">
-        <v>389.7693</v>
+        <v>241.8951</v>
       </c>
       <c r="E288" s="11" t="n">
-        <v>88.09699999999999</v>
+        <v>67.53570000000001</v>
       </c>
       <c r="F288" s="11" t="n">
-        <v>11.903</v>
+        <v>32.4643</v>
       </c>
       <c r="G288" s="11" t="n">
-        <v>-2.8134</v>
+        <v>-2.7469</v>
       </c>
       <c r="H288" s="11" t="n">
-        <v>47.6768</v>
+        <v>49.5968</v>
       </c>
       <c r="I288" s="11" t="n">
-        <v>0.4639</v>
+        <v>0.4685</v>
       </c>
       <c r="J288" s="11" t="n">
-        <v>0.9381</v>
+        <v>0.9369</v>
       </c>
       <c r="K288" s="11" t="n">
-        <v>0.6208</v>
+        <v>0.6246</v>
       </c>
     </row>
     <row r="289">
@@ -11889,31 +11889,31 @@
         </is>
       </c>
       <c r="C290" s="3" t="n">
-        <v>605.2036000000001</v>
+        <v>637.1436</v>
       </c>
       <c r="D290" s="3" t="n">
-        <v>472.6574</v>
+        <v>509.0637</v>
       </c>
       <c r="E290" s="3" t="n">
-        <v>4.0213</v>
+        <v>4.3751</v>
       </c>
       <c r="F290" s="3" t="n">
-        <v>95.9787</v>
+        <v>95.6249</v>
       </c>
       <c r="G290" s="3" t="n">
-        <v>-0.0351</v>
+        <v>-0.2574</v>
       </c>
       <c r="H290" s="3" t="n">
-        <v>53.9394</v>
+        <v>53.2258</v>
       </c>
       <c r="I290" s="3" t="n">
-        <v>0.5351</v>
+        <v>0.512</v>
       </c>
       <c r="J290" s="3" t="n">
-        <v>0.5</v>
+        <v>0.7083</v>
       </c>
       <c r="K290" s="3" t="n">
-        <v>0.5169</v>
+        <v>0.5944</v>
       </c>
     </row>
     <row r="291">
@@ -12045,31 +12045,31 @@
         </is>
       </c>
       <c r="C294" s="11" t="n">
-        <v>596.5811</v>
+        <v>582.8566</v>
       </c>
       <c r="D294" s="11" t="n">
-        <v>470.4259</v>
+        <v>462.9263</v>
       </c>
       <c r="E294" s="11" t="n">
-        <v>4.0248</v>
+        <v>3.9552</v>
       </c>
       <c r="F294" s="11" t="n">
-        <v>95.9752</v>
+        <v>96.0448</v>
       </c>
       <c r="G294" s="11" t="n">
-        <v>-0.0058</v>
+        <v>-0.0523</v>
       </c>
       <c r="H294" s="11" t="n">
-        <v>53.5354</v>
+        <v>56.0484</v>
       </c>
       <c r="I294" s="11" t="n">
-        <v>0.5271</v>
+        <v>0.5369</v>
       </c>
       <c r="J294" s="11" t="n">
-        <v>0.5574</v>
+        <v>0.6667</v>
       </c>
       <c r="K294" s="11" t="n">
-        <v>0.5417999999999999</v>
+        <v>0.5948</v>
       </c>
     </row>
     <row r="295">
@@ -12123,31 +12123,31 @@
         </is>
       </c>
       <c r="C296" s="3" t="n">
-        <v>31.1329</v>
+        <v>40.4235</v>
       </c>
       <c r="D296" s="3" t="n">
-        <v>23.1757</v>
+        <v>31.7792</v>
       </c>
       <c r="E296" s="3" t="n">
-        <v>10.5095</v>
+        <v>15.708</v>
       </c>
       <c r="F296" s="3" t="n">
-        <v>89.4905</v>
+        <v>84.292</v>
       </c>
       <c r="G296" s="3" t="n">
-        <v>-0.1721</v>
+        <v>-1.4866</v>
       </c>
       <c r="H296" s="3" t="n">
-        <v>52.7273</v>
+        <v>48.3871</v>
       </c>
       <c r="I296" s="3" t="n">
-        <v>0.5089</v>
+        <v>0.4739</v>
       </c>
       <c r="J296" s="3" t="n">
-        <v>0.7167</v>
+        <v>0.9397</v>
       </c>
       <c r="K296" s="3" t="n">
-        <v>0.5952</v>
+        <v>0.6301</v>
       </c>
     </row>
     <row r="297">
@@ -12279,31 +12279,31 @@
         </is>
       </c>
       <c r="C300" s="11" t="n">
-        <v>31.4959</v>
+        <v>40.5057</v>
       </c>
       <c r="D300" s="11" t="n">
-        <v>23.5367</v>
+        <v>31.8694</v>
       </c>
       <c r="E300" s="11" t="n">
-        <v>10.6897</v>
+        <v>15.7498</v>
       </c>
       <c r="F300" s="11" t="n">
-        <v>89.3103</v>
+        <v>84.25020000000001</v>
       </c>
       <c r="G300" s="11" t="n">
-        <v>-0.1996</v>
+        <v>-1.4967</v>
       </c>
       <c r="H300" s="11" t="n">
-        <v>52.9293</v>
+        <v>48.7903</v>
       </c>
       <c r="I300" s="11" t="n">
-        <v>0.5101</v>
+        <v>0.476</v>
       </c>
       <c r="J300" s="11" t="n">
-        <v>0.7375</v>
+        <v>0.9397</v>
       </c>
       <c r="K300" s="11" t="n">
-        <v>0.6031</v>
+        <v>0.6319</v>
       </c>
     </row>
     <row r="301">
@@ -14208,31 +14208,31 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>376.7233</v>
+        <v>311.4102</v>
       </c>
       <c r="C2" s="24" t="n">
-        <v>310.5403</v>
+        <v>260.3912</v>
       </c>
       <c r="D2" s="24" t="n">
-        <v>14.5269</v>
+        <v>11.0469</v>
       </c>
       <c r="E2" s="24" t="n">
-        <v>85.4731</v>
+        <v>88.95310000000001</v>
       </c>
       <c r="F2" s="24" t="n">
-        <v>-1.2876</v>
+        <v>-1.1632</v>
       </c>
       <c r="G2" s="24" t="n">
-        <v>51.103</v>
+        <v>50.75</v>
       </c>
       <c r="H2" s="24" t="n">
-        <v>0.5256999999999999</v>
+        <v>0.5347</v>
       </c>
       <c r="I2" s="24" t="n">
-        <v>0.4804</v>
+        <v>0.5118</v>
       </c>
       <c r="J2" s="24" t="n">
-        <v>0.4318</v>
+        <v>0.4502</v>
       </c>
     </row>
     <row r="3">
@@ -14242,31 +14242,31 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>376.7821</v>
+        <v>310.641</v>
       </c>
       <c r="C3" s="24" t="n">
-        <v>310.9717</v>
+        <v>259.8228</v>
       </c>
       <c r="D3" s="24" t="n">
-        <v>14.5954</v>
+        <v>11.0606</v>
       </c>
       <c r="E3" s="24" t="n">
-        <v>85.4046</v>
+        <v>88.93940000000001</v>
       </c>
       <c r="F3" s="24" t="n">
-        <v>-1.3161</v>
+        <v>-1.1649</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>51.1677</v>
+        <v>50.7097</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>0.5256</v>
+        <v>0.5365</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>0.4807</v>
+        <v>0.5118</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>0.4295</v>
+        <v>0.4495</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Update report template and charts to highlight ARIMA-LSTM as champion
</commit_message>
<xml_diff>
--- a/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
+++ b/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="All Models All Stocks" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CNN-LSTM Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ARIMA-LSTM Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Model Average Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -47,7 +47,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -94,21 +94,6 @@
         <fgColor rgb="00C8EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEBEE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -175,24 +160,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -12426,1701 +12393,1701 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>93.73569999999999</v>
+        <v>17.6343</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>72.3232</v>
+        <v>9.5032</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>2.3375</v>
+        <v>1.5902</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>97.66249999999999</v>
+        <v>98.4098</v>
       </c>
       <c r="F2" s="16" t="n">
-        <v>0.9743000000000001</v>
+        <v>0.994</v>
       </c>
       <c r="G2" s="16" t="n">
-        <v>47.3573</v>
+        <v>45.749</v>
       </c>
       <c r="H2" s="16" t="n">
-        <v>0.4441</v>
+        <v>0.4559</v>
       </c>
       <c r="I2" s="16" t="n">
-        <v>0.7381</v>
+        <v>0.9602000000000001</v>
       </c>
       <c r="J2" s="16" t="n">
-        <v>0.5546</v>
+        <v>0.6182</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>10.4736</v>
+        <v>47.1907</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>7.5056</v>
+        <v>32.4841</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>2.008</v>
+        <v>1.0297</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>97.992</v>
+        <v>98.97029999999999</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>0.9573</v>
+        <v>0.9937</v>
       </c>
       <c r="G3" s="16" t="n">
-        <v>53.0655</v>
+        <v>55.0607</v>
       </c>
       <c r="H3" s="16" t="n">
-        <v>0.4954</v>
+        <v>0</v>
       </c>
       <c r="I3" s="16" t="n">
-        <v>0.4864</v>
+        <v>0</v>
       </c>
       <c r="J3" s="16" t="n">
-        <v>0.4908</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>6.0728</v>
+        <v>4.4523</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>4.5734</v>
+        <v>3.0734</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1.9455</v>
+        <v>0.8184</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>98.0545</v>
+        <v>99.1816</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>0.957</v>
+        <v>0.9923</v>
       </c>
       <c r="G4" s="16" t="n">
-        <v>49.4715</v>
+        <v>54.0486</v>
       </c>
       <c r="H4" s="16" t="n">
-        <v>0.4926</v>
+        <v>0.6</v>
       </c>
       <c r="I4" s="16" t="n">
-        <v>0.7137</v>
+        <v>0.0391</v>
       </c>
       <c r="J4" s="16" t="n">
-        <v>0.5829</v>
+        <v>0.0735</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>5.2964</v>
+        <v>101.6614</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>4.0139</v>
+        <v>70.3026</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>2.4619</v>
+        <v>1.1654</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>97.5381</v>
+        <v>98.83459999999999</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>0.9546</v>
+        <v>0.9912</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>49.26</v>
+        <v>50</v>
       </c>
       <c r="H5" s="16" t="n">
-        <v>0.5081</v>
+        <v>0.5714</v>
       </c>
       <c r="I5" s="16" t="n">
-        <v>0.5123</v>
+        <v>0.0161</v>
       </c>
       <c r="J5" s="16" t="n">
-        <v>0.5102</v>
+        <v>0.0314</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>40.8654</v>
+        <v>14.378</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>27.7295</v>
+        <v>10.3798</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>3.1896</v>
+        <v>1.3492</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>96.8104</v>
+        <v>98.6508</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.9532</v>
+        <v>0.9907</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>52.2199</v>
+        <v>54.6559</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>0.518</v>
+        <v>0.5504</v>
       </c>
       <c r="I6" s="16" t="n">
-        <v>0.6102</v>
+        <v>0.9296</v>
       </c>
       <c r="J6" s="16" t="n">
-        <v>0.5603</v>
+        <v>0.6915</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>LTM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>161.346</v>
+        <v>17.2348</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>126.4788</v>
+        <v>12.1314</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>2.4627</v>
+        <v>1.662</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>97.5373</v>
+        <v>98.33799999999999</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>0.9512</v>
+        <v>0.9898</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>50.9554</v>
+        <v>50.4049</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>0.5248</v>
+        <v>0.509</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>0.4398</v>
+        <v>0.7857</v>
       </c>
       <c r="J7" s="16" t="n">
-        <v>0.4786</v>
+        <v>0.6178</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>47.1562</v>
+        <v>12.7136</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>32.2792</v>
+        <v>8.7629</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>5.7555</v>
+        <v>1.0076</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>94.2445</v>
+        <v>98.9924</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>0.9510999999999999</v>
+        <v>0.9897</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>48.6258</v>
+        <v>51.2146</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0.4694</v>
+        <v>0.5125999999999999</v>
       </c>
       <c r="I8" s="16" t="n">
-        <v>0.8401999999999999</v>
+        <v>0.9684</v>
       </c>
       <c r="J8" s="16" t="n">
-        <v>0.6022999999999999</v>
+        <v>0.6703</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>165.3966</v>
+        <v>22.3796</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>125.2871</v>
+        <v>13.2825</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>2.5457</v>
+        <v>1.4713</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>97.4543</v>
+        <v>98.5287</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9885</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>50.3171</v>
+        <v>48.7854</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>0.5115</v>
+        <v>0.4898</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>0.3724</v>
+        <v>0.9918</v>
       </c>
       <c r="J9" s="16" t="n">
-        <v>0.431</v>
+        <v>0.6558</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>16.8316</v>
+        <v>188.8798</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>13.3532</v>
+        <v>135.2834</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>1.9233</v>
+        <v>1.0233</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>98.0767</v>
+        <v>98.97669999999999</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.9449</v>
+        <v>0.9878</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>52.5926</v>
+        <v>51.6194</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.4836</v>
+        <v>0.6471</v>
       </c>
       <c r="I10" s="16" t="n">
-        <v>0.3138</v>
+        <v>0.0451</v>
       </c>
       <c r="J10" s="16" t="n">
-        <v>0.3806</v>
+        <v>0.0843</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>58.147</v>
+        <v>78.49290000000001</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>44.8118</v>
+        <v>59.2656</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>2.8562</v>
+        <v>1.2414</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>97.1438</v>
+        <v>98.7586</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>0.9306</v>
+        <v>0.9876</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>52.0085</v>
+        <v>55.0607</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>0.5304</v>
+        <v>0.5461</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>0.2607</v>
+        <v>0.6425999999999999</v>
       </c>
       <c r="J11" s="16" t="n">
-        <v>0.3496</v>
+        <v>0.5904</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>136.9449</v>
+        <v>23.3457</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>100.3581</v>
+        <v>17.1383</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>1.8297</v>
+        <v>0.9863</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>98.1703</v>
+        <v>99.0137</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.9089</v>
+        <v>0.9865</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>53.4884</v>
+        <v>50.2315</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.4845</v>
       </c>
       <c r="I12" s="16" t="n">
-        <v>0.5595</v>
+        <v>0.2217</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>0.5618</v>
+        <v>0.3042</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>2.8438</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>2.0466</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>1.2722</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>98.7278</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>0.9864000000000001</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>53.2389</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>0.5331</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>0.6414</v>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>0.5823</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>25.663</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>18.4288</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>1.2383</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>98.7617</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>0.9863</v>
+      </c>
+      <c r="G14" s="16" t="n">
+        <v>46.5587</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>0.4586</v>
+      </c>
+      <c r="I14" s="16" t="n">
+        <v>0.5041</v>
+      </c>
+      <c r="J14" s="16" t="n">
+        <v>0.4803</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>35.7489</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>25.7072</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>1.0216</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>98.97839999999999</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>0.9852</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>51.8219</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>0.0206</v>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>0.0403</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>23.2492</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>17.2364</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>0.9638</v>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>99.03619999999999</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>0.9846</v>
+      </c>
+      <c r="G16" s="16" t="n">
+        <v>51.2146</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="I16" s="16" t="n">
+        <v>0.8611</v>
+      </c>
+      <c r="J16" s="16" t="n">
+        <v>0.643</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>15.1184</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>10.9335</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>1.2685</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>98.7315</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>0.9843</v>
+      </c>
+      <c r="G17" s="16" t="n">
+        <v>48.3806</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>10.4175</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>7.7411</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>0.9043</v>
+      </c>
+      <c r="E18" s="16" t="n">
+        <v>99.09569999999999</v>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>0.9826</v>
+      </c>
+      <c r="G18" s="16" t="n">
+        <v>51.8219</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>0.5143</v>
+      </c>
+      <c r="I18" s="16" t="n">
+        <v>0.07530000000000001</v>
+      </c>
+      <c r="J18" s="16" t="n">
+        <v>0.1314</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="n">
+        <v>16.4069</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>11.9738</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>1.1346</v>
+      </c>
+      <c r="E19" s="16" t="n">
+        <v>98.86539999999999</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>0.9814000000000001</v>
+      </c>
+      <c r="G19" s="16" t="n">
+        <v>51.0121</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>0.5192</v>
+      </c>
+      <c r="I19" s="16" t="n">
+        <v>0.6378</v>
+      </c>
+      <c r="J19" s="16" t="n">
+        <v>0.5724</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>9.8278</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>7.6279</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <v>1.119</v>
+      </c>
+      <c r="E20" s="16" t="n">
+        <v>98.881</v>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>0.9804</v>
+      </c>
+      <c r="G20" s="16" t="n">
+        <v>45.5399</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>0.4554</v>
+      </c>
+      <c r="I20" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="16" t="n">
+        <v>0.6258</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="n">
+        <v>100.6076</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>72.4442</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>1.4308</v>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>98.5692</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>0.9802999999999999</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>50.2033</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>0.5011</v>
+      </c>
+      <c r="I21" s="16" t="n">
+        <v>0.9146</v>
+      </c>
+      <c r="J21" s="16" t="n">
+        <v>0.6475</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>25.0713</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>17.1767</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <v>1.1522</v>
+      </c>
+      <c r="E22" s="16" t="n">
+        <v>98.84780000000001</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>0.9802999999999999</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <v>47.7733</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>0.4635</v>
+      </c>
+      <c r="I22" s="16" t="n">
+        <v>0.5336</v>
+      </c>
+      <c r="J22" s="16" t="n">
+        <v>0.4961</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="n">
+        <v>54.5999</v>
+      </c>
+      <c r="C23" s="16" t="n">
+        <v>38.4763</v>
+      </c>
+      <c r="D23" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="E23" s="16" t="n">
+        <v>98.95480000000001</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>0.9802999999999999</v>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>51.417</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>0.5105</v>
+      </c>
+      <c r="I23" s="16" t="n">
+        <v>0.6883</v>
+      </c>
+      <c r="J23" s="16" t="n">
+        <v>0.5862000000000001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>26.2286</v>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>19.1449</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>1.3974</v>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>98.6026</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>0.9792999999999999</v>
+      </c>
+      <c r="G24" s="16" t="n">
+        <v>46.1538</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <v>0.4699</v>
+      </c>
+      <c r="I24" s="16" t="n">
+        <v>0.9536</v>
+      </c>
+      <c r="J24" s="16" t="n">
+        <v>0.6294999999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>4.2772</v>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>3.0455</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>1.261</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>98.739</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>0.9779</v>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>51.2146</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <v>0.4857</v>
+      </c>
+      <c r="I25" s="16" t="n">
+        <v>0.0708</v>
+      </c>
+      <c r="J25" s="16" t="n">
+        <v>0.1236</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>15.1073</v>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>10.9683</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>0.9019</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <v>99.0981</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>0.9777</v>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>49.1903</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <v>0.4906</v>
+      </c>
+      <c r="I26" s="16" t="n">
+        <v>0.6367</v>
+      </c>
+      <c r="J26" s="16" t="n">
+        <v>0.5542</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>6.1831</v>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>4.4508</v>
+      </c>
+      <c r="D27" s="16" t="n">
+        <v>1.1012</v>
+      </c>
+      <c r="E27" s="16" t="n">
+        <v>98.89879999999999</v>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>0.9772</v>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>51.0121</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <v>0.5101</v>
+      </c>
+      <c r="I27" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="16" t="n">
+        <v>0.6756</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>151.642</v>
+      </c>
+      <c r="C28" s="16" t="n">
+        <v>105.8179</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <v>1.1703</v>
+      </c>
+      <c r="E28" s="16" t="n">
+        <v>98.8297</v>
+      </c>
+      <c r="F28" s="16" t="n">
+        <v>0.9752</v>
+      </c>
+      <c r="G28" s="16" t="n">
+        <v>51.0121</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="I28" s="16" t="n">
+        <v>0.9249000000000001</v>
+      </c>
+      <c r="J28" s="16" t="n">
+        <v>0.6592</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="n">
+        <v>5.5735</v>
+      </c>
+      <c r="C29" s="16" t="n">
+        <v>4.1427</v>
+      </c>
+      <c r="D29" s="16" t="n">
+        <v>1.3725</v>
+      </c>
+      <c r="E29" s="16" t="n">
+        <v>98.6275</v>
+      </c>
+      <c r="F29" s="16" t="n">
+        <v>0.9746</v>
+      </c>
+      <c r="G29" s="16" t="n">
+        <v>47.9757</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <v>0.4783</v>
+      </c>
+      <c r="I29" s="16" t="n">
+        <v>0.9788</v>
+      </c>
+      <c r="J29" s="16" t="n">
+        <v>0.6425999999999999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>71.2376</v>
+      </c>
+      <c r="C30" s="16" t="n">
+        <v>52.1747</v>
+      </c>
+      <c r="D30" s="16" t="n">
+        <v>0.9447</v>
+      </c>
+      <c r="E30" s="16" t="n">
+        <v>99.0553</v>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="G30" s="16" t="n">
+        <v>52.834</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <v>0.5283</v>
+      </c>
+      <c r="I30" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="16" t="n">
+        <v>0.6914</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>4.9786</v>
+      </c>
+      <c r="C31" s="16" t="n">
+        <v>3.7878</v>
+      </c>
+      <c r="D31" s="16" t="n">
+        <v>1.0757</v>
+      </c>
+      <c r="E31" s="16" t="n">
+        <v>98.9243</v>
+      </c>
+      <c r="F31" s="16" t="n">
+        <v>0.9733000000000001</v>
+      </c>
+      <c r="G31" s="16" t="n">
+        <v>49.7976</v>
+      </c>
+      <c r="H31" s="16" t="n">
+        <v>0.4706</v>
+      </c>
+      <c r="I31" s="16" t="n">
+        <v>0.2667</v>
+      </c>
+      <c r="J31" s="16" t="n">
+        <v>0.3404</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="n">
+        <v>29.7503</v>
+      </c>
+      <c r="C32" s="16" t="n">
+        <v>21.8678</v>
+      </c>
+      <c r="D32" s="16" t="n">
+        <v>0.9267</v>
+      </c>
+      <c r="E32" s="16" t="n">
+        <v>99.0733</v>
+      </c>
+      <c r="F32" s="16" t="n">
+        <v>0.9725</v>
+      </c>
+      <c r="G32" s="16" t="n">
+        <v>48.583</v>
+      </c>
+      <c r="H32" s="16" t="n">
+        <v>0.4787</v>
+      </c>
+      <c r="I32" s="16" t="n">
+        <v>0.9615</v>
+      </c>
+      <c r="J32" s="16" t="n">
+        <v>0.6392</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>17.4161</v>
+      </c>
+      <c r="C33" s="16" t="n">
+        <v>12.3129</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <v>1.0319</v>
+      </c>
+      <c r="E33" s="16" t="n">
+        <v>98.96810000000001</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>0.9711</v>
+      </c>
+      <c r="G33" s="16" t="n">
+        <v>53.4413</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <v>0.5266</v>
+      </c>
+      <c r="I33" s="16" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="J33" s="16" t="n">
+        <v>0.4626</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="n">
+        <v>93.0487</v>
+      </c>
+      <c r="C34" s="16" t="n">
+        <v>66.62390000000001</v>
+      </c>
+      <c r="D34" s="16" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="E34" s="16" t="n">
+        <v>99.074</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <v>51.0121</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I34" s="16" t="n">
+        <v>0.7355</v>
+      </c>
+      <c r="J34" s="16" t="n">
+        <v>0.5953000000000001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="n">
+        <v>54.9985</v>
+      </c>
+      <c r="C35" s="16" t="n">
+        <v>42.3928</v>
+      </c>
+      <c r="D35" s="16" t="n">
+        <v>1.3882</v>
+      </c>
+      <c r="E35" s="16" t="n">
+        <v>98.6118</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>51.417</v>
+      </c>
+      <c r="H35" s="16" t="n">
+        <v>0.5197000000000001</v>
+      </c>
+      <c r="I35" s="16" t="n">
+        <v>0.5777</v>
+      </c>
+      <c r="J35" s="16" t="n">
+        <v>0.5472</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>95.30670000000001</v>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>68.5162</v>
+      </c>
+      <c r="D36" s="16" t="n">
+        <v>1.1395</v>
+      </c>
+      <c r="E36" s="16" t="n">
+        <v>98.8605</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <v>0.9693000000000001</v>
+      </c>
+      <c r="G36" s="16" t="n">
+        <v>45.6389</v>
+      </c>
+      <c r="H36" s="16" t="n">
+        <v>0.4608</v>
+      </c>
+      <c r="I36" s="16" t="n">
+        <v>0.3984</v>
+      </c>
+      <c r="J36" s="16" t="n">
+        <v>0.4274</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>28.8329</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>21.5165</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <v>1.1564</v>
+      </c>
+      <c r="E37" s="16" t="n">
+        <v>98.8436</v>
+      </c>
+      <c r="F37" s="16" t="n">
+        <v>0.9678</v>
+      </c>
+      <c r="G37" s="16" t="n">
+        <v>50.8097</v>
+      </c>
+      <c r="H37" s="16" t="n">
+        <v>0.5714</v>
+      </c>
+      <c r="I37" s="16" t="n">
+        <v>0.0327</v>
+      </c>
+      <c r="J37" s="16" t="n">
+        <v>0.0618</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="n">
+        <v>4.348</v>
+      </c>
+      <c r="C38" s="16" t="n">
+        <v>3.1116</v>
+      </c>
+      <c r="D38" s="16" t="n">
+        <v>1.2428</v>
+      </c>
+      <c r="E38" s="16" t="n">
+        <v>98.7572</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>0.9678</v>
+      </c>
+      <c r="G38" s="16" t="n">
+        <v>45.5466</v>
+      </c>
+      <c r="H38" s="16" t="n">
+        <v>0.4659</v>
+      </c>
+      <c r="I38" s="16" t="n">
+        <v>0.8577</v>
+      </c>
+      <c r="J38" s="16" t="n">
+        <v>0.6038</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="n">
+        <v>17.8948</v>
+      </c>
+      <c r="C39" s="16" t="n">
+        <v>13.3063</v>
+      </c>
+      <c r="D39" s="16" t="n">
+        <v>0.9741</v>
+      </c>
+      <c r="E39" s="16" t="n">
+        <v>99.02589999999999</v>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>0.9676</v>
+      </c>
+      <c r="G39" s="16" t="n">
+        <v>49.5951</v>
+      </c>
+      <c r="H39" s="16" t="n">
+        <v>0.4928</v>
+      </c>
+      <c r="I39" s="16" t="n">
+        <v>0.9876</v>
+      </c>
+      <c r="J39" s="16" t="n">
+        <v>0.6575</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
           <t>ADANIENT</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
-        <v>100.3856</v>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>75.27930000000001</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>96.91</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>0.9009</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>46.723</v>
-      </c>
-      <c r="H13" s="16" t="n">
-        <v>0.4537</v>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>0.6368</v>
-      </c>
-      <c r="J13" s="16" t="n">
-        <v>0.5299</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="n">
-        <v>90.7525</v>
-      </c>
-      <c r="C14" s="18" t="n">
-        <v>72.5277</v>
-      </c>
-      <c r="D14" s="18" t="n">
-        <v>2.937</v>
-      </c>
-      <c r="E14" s="18" t="n">
-        <v>97.063</v>
-      </c>
-      <c r="F14" s="18" t="n">
-        <v>0.8998</v>
-      </c>
-      <c r="G14" s="18" t="n">
-        <v>50.74</v>
-      </c>
-      <c r="H14" s="18" t="n">
-        <v>0.5013</v>
-      </c>
-      <c r="I14" s="18" t="n">
-        <v>0.8462</v>
-      </c>
-      <c r="J14" s="18" t="n">
-        <v>0.6296</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>ONGC</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>7.2512</v>
-      </c>
-      <c r="C15" s="18" t="n">
-        <v>5.4998</v>
-      </c>
-      <c r="D15" s="18" t="n">
-        <v>2.2068</v>
-      </c>
-      <c r="E15" s="18" t="n">
-        <v>97.7932</v>
-      </c>
-      <c r="F15" s="18" t="n">
-        <v>0.8985</v>
-      </c>
-      <c r="G15" s="18" t="n">
-        <v>54.1226</v>
-      </c>
-      <c r="H15" s="18" t="n">
-        <v>0.5385</v>
-      </c>
-      <c r="I15" s="18" t="n">
-        <v>0.3668</v>
-      </c>
-      <c r="J15" s="18" t="n">
-        <v>0.4364</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>AXISBANK</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="n">
-        <v>34.0067</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <v>25.9482</v>
-      </c>
-      <c r="D16" s="18" t="n">
-        <v>2.1327</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>97.8673</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>0.8921</v>
-      </c>
-      <c r="G16" s="18" t="n">
-        <v>51.797</v>
-      </c>
-      <c r="H16" s="18" t="n">
-        <v>0.5276</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>0.2851</v>
-      </c>
-      <c r="J16" s="18" t="n">
-        <v>0.3702</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="B40" s="16" t="n">
+        <v>62.2551</v>
+      </c>
+      <c r="C40" s="16" t="n">
+        <v>41.9635</v>
+      </c>
+      <c r="D40" s="16" t="n">
+        <v>1.718</v>
+      </c>
+      <c r="E40" s="16" t="n">
+        <v>98.282</v>
+      </c>
+      <c r="F40" s="16" t="n">
+        <v>0.9655</v>
+      </c>
+      <c r="G40" s="16" t="n">
+        <v>46.5587</v>
+      </c>
+      <c r="H40" s="16" t="n">
+        <v>0.4619</v>
+      </c>
+      <c r="I40" s="16" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="J40" s="16" t="n">
+        <v>0.6024</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="n">
+        <v>5.5064</v>
+      </c>
+      <c r="C41" s="16" t="n">
+        <v>3.9313</v>
+      </c>
+      <c r="D41" s="16" t="n">
+        <v>0.9984</v>
+      </c>
+      <c r="E41" s="16" t="n">
+        <v>99.0016</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <v>0.9653</v>
+      </c>
+      <c r="G41" s="16" t="n">
+        <v>47.7733</v>
+      </c>
+      <c r="H41" s="16" t="n">
+        <v>0.4813</v>
+      </c>
+      <c r="I41" s="16" t="n">
+        <v>0.9667</v>
+      </c>
+      <c r="J41" s="16" t="n">
+        <v>0.6427</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>TATACONSUM</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n">
-        <v>29.7318</v>
-      </c>
-      <c r="C17" s="18" t="n">
-        <v>22.7336</v>
-      </c>
-      <c r="D17" s="18" t="n">
-        <v>2.1379</v>
-      </c>
-      <c r="E17" s="18" t="n">
-        <v>97.8621</v>
-      </c>
-      <c r="F17" s="18" t="n">
-        <v>0.8782</v>
-      </c>
-      <c r="G17" s="18" t="n">
-        <v>55.814</v>
-      </c>
-      <c r="H17" s="18" t="n">
-        <v>0.5486</v>
-      </c>
-      <c r="I17" s="18" t="n">
-        <v>0.6026</v>
-      </c>
-      <c r="J17" s="18" t="n">
-        <v>0.5743</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="B42" s="16" t="n">
+        <v>15.9316</v>
+      </c>
+      <c r="C42" s="16" t="n">
+        <v>11.6284</v>
+      </c>
+      <c r="D42" s="16" t="n">
+        <v>1.0718</v>
+      </c>
+      <c r="E42" s="16" t="n">
+        <v>98.9282</v>
+      </c>
+      <c r="F42" s="16" t="n">
+        <v>0.9651</v>
+      </c>
+      <c r="G42" s="16" t="n">
+        <v>53.8462</v>
+      </c>
+      <c r="H42" s="16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I42" s="16" t="n">
+        <v>0.1736</v>
+      </c>
+      <c r="J42" s="16" t="n">
+        <v>0.2692</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="n">
+        <v>15.3081</v>
+      </c>
+      <c r="C43" s="16" t="n">
+        <v>11.3317</v>
+      </c>
+      <c r="D43" s="16" t="n">
+        <v>0.8598</v>
+      </c>
+      <c r="E43" s="16" t="n">
+        <v>99.14019999999999</v>
+      </c>
+      <c r="F43" s="16" t="n">
+        <v>0.9651</v>
+      </c>
+      <c r="G43" s="16" t="n">
+        <v>51.6194</v>
+      </c>
+      <c r="H43" s="16" t="n">
+        <v>0.509</v>
+      </c>
+      <c r="I43" s="16" t="n">
+        <v>0.6898</v>
+      </c>
+      <c r="J43" s="16" t="n">
+        <v>0.5858</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="n">
+        <v>56.7748</v>
+      </c>
+      <c r="C44" s="16" t="n">
+        <v>39.3751</v>
+      </c>
+      <c r="D44" s="16" t="n">
+        <v>1.0852</v>
+      </c>
+      <c r="E44" s="16" t="n">
+        <v>98.9148</v>
+      </c>
+      <c r="F44" s="16" t="n">
+        <v>0.9589</v>
+      </c>
+      <c r="G44" s="16" t="n">
+        <v>48.3806</v>
+      </c>
+      <c r="H44" s="16" t="n">
+        <v>0.4573</v>
+      </c>
+      <c r="I44" s="16" t="n">
+        <v>0.3824</v>
+      </c>
+      <c r="J44" s="16" t="n">
+        <v>0.4165</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="n">
+        <v>4.1778</v>
+      </c>
+      <c r="C45" s="16" t="n">
+        <v>3.0856</v>
+      </c>
+      <c r="D45" s="16" t="n">
+        <v>1.0621</v>
+      </c>
+      <c r="E45" s="16" t="n">
+        <v>98.9379</v>
+      </c>
+      <c r="F45" s="16" t="n">
+        <v>0.9577</v>
+      </c>
+      <c r="G45" s="16" t="n">
+        <v>48.583</v>
+      </c>
+      <c r="H45" s="16" t="n">
+        <v>0.4774</v>
+      </c>
+      <c r="I45" s="16" t="n">
+        <v>0.5685</v>
+      </c>
+      <c r="J45" s="16" t="n">
+        <v>0.5189</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="n">
+        <v>38.1726</v>
+      </c>
+      <c r="C46" s="16" t="n">
+        <v>28.0103</v>
+      </c>
+      <c r="D46" s="16" t="n">
+        <v>1.0385</v>
+      </c>
+      <c r="E46" s="16" t="n">
+        <v>98.9615</v>
+      </c>
+      <c r="F46" s="16" t="n">
+        <v>0.9542</v>
+      </c>
+      <c r="G46" s="16" t="n">
+        <v>46.1538</v>
+      </c>
+      <c r="H46" s="16" t="n">
+        <v>0.4561</v>
+      </c>
+      <c r="I46" s="16" t="n">
+        <v>0.5394</v>
+      </c>
+      <c r="J46" s="16" t="n">
+        <v>0.4943</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>CIPLA</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n">
-        <v>33.2858</v>
-      </c>
-      <c r="C18" s="18" t="n">
-        <v>26.1273</v>
-      </c>
-      <c r="D18" s="18" t="n">
-        <v>1.7969</v>
-      </c>
-      <c r="E18" s="18" t="n">
-        <v>98.20310000000001</v>
-      </c>
-      <c r="F18" s="18" t="n">
-        <v>0.8774999999999999</v>
-      </c>
-      <c r="G18" s="18" t="n">
-        <v>48.4144</v>
-      </c>
-      <c r="H18" s="18" t="n">
-        <v>0.4952</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>0.4256</v>
-      </c>
-      <c r="J18" s="18" t="n">
-        <v>0.4578</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>HCLTECH</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="n">
-        <v>64.92189999999999</v>
-      </c>
-      <c r="C19" s="18" t="n">
-        <v>52.2882</v>
-      </c>
-      <c r="D19" s="18" t="n">
-        <v>3.4071</v>
-      </c>
-      <c r="E19" s="18" t="n">
-        <v>96.5929</v>
-      </c>
-      <c r="F19" s="18" t="n">
-        <v>0.873</v>
-      </c>
-      <c r="G19" s="18" t="n">
-        <v>47.5687</v>
-      </c>
-      <c r="H19" s="18" t="n">
-        <v>0.4234</v>
-      </c>
-      <c r="I19" s="18" t="n">
-        <v>0.2035</v>
-      </c>
-      <c r="J19" s="18" t="n">
-        <v>0.2749</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>ADANIPORTS</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="n">
-        <v>68.7503</v>
-      </c>
-      <c r="C20" s="18" t="n">
-        <v>56.3474</v>
-      </c>
-      <c r="D20" s="18" t="n">
-        <v>4.0657</v>
-      </c>
-      <c r="E20" s="18" t="n">
-        <v>95.93429999999999</v>
-      </c>
-      <c r="F20" s="18" t="n">
-        <v>0.8616</v>
-      </c>
-      <c r="G20" s="18" t="n">
-        <v>48.203</v>
-      </c>
-      <c r="H20" s="18" t="n">
-        <v>0.479</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>0.7435</v>
-      </c>
-      <c r="J20" s="18" t="n">
-        <v>0.5826</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>HINDALCO</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="n">
-        <v>57.5723</v>
-      </c>
-      <c r="C21" s="18" t="n">
-        <v>39.8599</v>
-      </c>
-      <c r="D21" s="18" t="n">
-        <v>4.5925</v>
-      </c>
-      <c r="E21" s="18" t="n">
-        <v>95.4075</v>
-      </c>
-      <c r="F21" s="18" t="n">
-        <v>0.8531</v>
-      </c>
-      <c r="G21" s="18" t="n">
-        <v>50.1057</v>
-      </c>
-      <c r="H21" s="18" t="n">
-        <v>0.6153999999999999</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>0.2738</v>
-      </c>
-      <c r="J21" s="18" t="n">
-        <v>0.3789</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>HINDUNILVR</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="n">
-        <v>69.70659999999999</v>
-      </c>
-      <c r="C22" s="18" t="n">
-        <v>55.7897</v>
-      </c>
-      <c r="D22" s="18" t="n">
-        <v>2.3058</v>
-      </c>
-      <c r="E22" s="18" t="n">
-        <v>97.6942</v>
-      </c>
-      <c r="F22" s="18" t="n">
-        <v>0.8435</v>
-      </c>
-      <c r="G22" s="18" t="n">
-        <v>52.8541</v>
-      </c>
-      <c r="H22" s="18" t="n">
-        <v>0.5132</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>0.1733</v>
-      </c>
-      <c r="J22" s="18" t="n">
-        <v>0.2591</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>MARUTI</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="n">
-        <v>725.0996</v>
-      </c>
-      <c r="C23" s="18" t="n">
-        <v>536.1033</v>
-      </c>
-      <c r="D23" s="18" t="n">
-        <v>3.7659</v>
-      </c>
-      <c r="E23" s="18" t="n">
-        <v>96.2341</v>
-      </c>
-      <c r="F23" s="18" t="n">
-        <v>0.8259</v>
-      </c>
-      <c r="G23" s="18" t="n">
-        <v>50.5285</v>
-      </c>
-      <c r="H23" s="18" t="n">
-        <v>0.5041</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>0.5169</v>
-      </c>
-      <c r="J23" s="18" t="n">
-        <v>0.5105</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="B47" s="16" t="n">
+        <v>20.368</v>
+      </c>
+      <c r="C47" s="16" t="n">
+        <v>14.2689</v>
+      </c>
+      <c r="D47" s="16" t="n">
+        <v>0.983</v>
+      </c>
+      <c r="E47" s="16" t="n">
+        <v>99.017</v>
+      </c>
+      <c r="F47" s="16" t="n">
+        <v>0.9526</v>
+      </c>
+      <c r="G47" s="16" t="n">
+        <v>50.8097</v>
+      </c>
+      <c r="H47" s="16" t="n">
+        <v>0.5073</v>
+      </c>
+      <c r="I47" s="16" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="J47" s="16" t="n">
+        <v>0.6676</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="B48" s="16" t="n">
+        <v>25.2575</v>
+      </c>
+      <c r="C48" s="16" t="n">
+        <v>19.0788</v>
+      </c>
+      <c r="D48" s="16" t="n">
+        <v>1.298</v>
+      </c>
+      <c r="E48" s="16" t="n">
+        <v>98.702</v>
+      </c>
+      <c r="F48" s="16" t="n">
+        <v>0.9394</v>
+      </c>
+      <c r="G48" s="16" t="n">
+        <v>48.7854</v>
+      </c>
+      <c r="H48" s="16" t="n">
+        <v>0.4895</v>
+      </c>
+      <c r="I48" s="16" t="n">
+        <v>0.9588</v>
+      </c>
+      <c r="J48" s="16" t="n">
+        <v>0.6481</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="n">
+        <v>21.533</v>
+      </c>
+      <c r="C49" s="16" t="n">
+        <v>15.6806</v>
+      </c>
+      <c r="D49" s="16" t="n">
+        <v>0.9135</v>
+      </c>
+      <c r="E49" s="16" t="n">
+        <v>99.0865</v>
+      </c>
+      <c r="F49" s="16" t="n">
+        <v>0.9337</v>
+      </c>
+      <c r="G49" s="16" t="n">
+        <v>52.834</v>
+      </c>
+      <c r="H49" s="16" t="n">
+        <v>0.5294</v>
+      </c>
+      <c r="I49" s="16" t="n">
+        <v>0.9962</v>
+      </c>
+      <c r="J49" s="16" t="n">
+        <v>0.6914</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>DRREDDY</t>
         </is>
       </c>
-      <c r="B24" s="18" t="n">
-        <v>26.806</v>
-      </c>
-      <c r="C24" s="18" t="n">
-        <v>21.0503</v>
-      </c>
-      <c r="D24" s="18" t="n">
-        <v>1.6797</v>
-      </c>
-      <c r="E24" s="18" t="n">
-        <v>98.3203</v>
-      </c>
-      <c r="F24" s="18" t="n">
-        <v>0.8216</v>
-      </c>
-      <c r="G24" s="18" t="n">
-        <v>51.5856</v>
-      </c>
-      <c r="H24" s="18" t="n">
-        <v>0.5272</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>0.4059</v>
-      </c>
-      <c r="J24" s="18" t="n">
-        <v>0.4586</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>HDFCBANK</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n">
-        <v>34.5244</v>
-      </c>
-      <c r="C25" s="18" t="n">
-        <v>28.7525</v>
-      </c>
-      <c r="D25" s="18" t="n">
-        <v>3.1601</v>
-      </c>
-      <c r="E25" s="18" t="n">
-        <v>96.8399</v>
-      </c>
-      <c r="F25" s="18" t="n">
-        <v>0.8058</v>
-      </c>
-      <c r="G25" s="18" t="n">
-        <v>52.4313</v>
-      </c>
-      <c r="H25" s="18" t="n">
-        <v>0.5221</v>
-      </c>
-      <c r="I25" s="18" t="n">
-        <v>0.3074</v>
-      </c>
-      <c r="J25" s="18" t="n">
-        <v>0.3869</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>SBILIFE</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="n">
-        <v>90.16589999999999</v>
-      </c>
-      <c r="C26" s="18" t="n">
-        <v>79.64919999999999</v>
-      </c>
-      <c r="D26" s="18" t="n">
-        <v>4.3847</v>
-      </c>
-      <c r="E26" s="18" t="n">
-        <v>95.6153</v>
-      </c>
-      <c r="F26" s="18" t="n">
-        <v>0.8055</v>
-      </c>
-      <c r="G26" s="18" t="n">
-        <v>50.2427</v>
-      </c>
-      <c r="H26" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>0.0146</v>
-      </c>
-      <c r="J26" s="18" t="n">
-        <v>0.0284</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>KOTAKBANK</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="n">
-        <v>12.99</v>
-      </c>
-      <c r="C27" s="18" t="n">
-        <v>10.6577</v>
-      </c>
-      <c r="D27" s="18" t="n">
-        <v>2.6112</v>
-      </c>
-      <c r="E27" s="18" t="n">
-        <v>97.3888</v>
-      </c>
-      <c r="F27" s="18" t="n">
-        <v>0.8015</v>
-      </c>
-      <c r="G27" s="18" t="n">
-        <v>53.0655</v>
-      </c>
-      <c r="H27" s="18" t="n">
-        <v>0.5926</v>
-      </c>
-      <c r="I27" s="18" t="n">
-        <v>0.2025</v>
-      </c>
-      <c r="J27" s="18" t="n">
-        <v>0.3019</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
-        <is>
-          <t>TECHM</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="n">
-        <v>47.2109</v>
-      </c>
-      <c r="C28" s="18" t="n">
-        <v>38.3846</v>
-      </c>
-      <c r="D28" s="18" t="n">
-        <v>2.5468</v>
-      </c>
-      <c r="E28" s="18" t="n">
-        <v>97.4532</v>
-      </c>
-      <c r="F28" s="18" t="n">
-        <v>0.792</v>
-      </c>
-      <c r="G28" s="18" t="n">
-        <v>50.5285</v>
-      </c>
-      <c r="H28" s="18" t="n">
-        <v>0.5145999999999999</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>0.2236</v>
-      </c>
-      <c r="J28" s="18" t="n">
-        <v>0.3118</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
-        <is>
-          <t>NESTLEIND</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="n">
-        <v>47.1488</v>
-      </c>
-      <c r="C29" s="18" t="n">
-        <v>35.4047</v>
-      </c>
-      <c r="D29" s="18" t="n">
-        <v>2.8102</v>
-      </c>
-      <c r="E29" s="18" t="n">
-        <v>97.18980000000001</v>
-      </c>
-      <c r="F29" s="18" t="n">
-        <v>0.7907</v>
-      </c>
-      <c r="G29" s="18" t="n">
-        <v>48.6258</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>0.3389</v>
-      </c>
-      <c r="J29" s="18" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B30" s="18" t="n">
-        <v>59.3728</v>
-      </c>
-      <c r="C30" s="18" t="n">
-        <v>40.388</v>
-      </c>
-      <c r="D30" s="18" t="n">
-        <v>4.1705</v>
-      </c>
-      <c r="E30" s="18" t="n">
-        <v>95.8295</v>
-      </c>
-      <c r="F30" s="18" t="n">
-        <v>0.7835</v>
-      </c>
-      <c r="G30" s="18" t="n">
-        <v>49.26</v>
-      </c>
-      <c r="H30" s="18" t="n">
-        <v>0.5333</v>
-      </c>
-      <c r="I30" s="18" t="n">
-        <v>0.2267</v>
-      </c>
-      <c r="J30" s="18" t="n">
-        <v>0.3182</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>GRASIM</t>
-        </is>
-      </c>
-      <c r="B31" s="18" t="n">
-        <v>87.05840000000001</v>
-      </c>
-      <c r="C31" s="18" t="n">
-        <v>69.8891</v>
-      </c>
-      <c r="D31" s="18" t="n">
-        <v>2.6108</v>
-      </c>
-      <c r="E31" s="18" t="n">
-        <v>97.3892</v>
-      </c>
-      <c r="F31" s="18" t="n">
-        <v>0.7694</v>
-      </c>
-      <c r="G31" s="18" t="n">
-        <v>50.74</v>
-      </c>
-      <c r="H31" s="18" t="n">
-        <v>0.5041</v>
-      </c>
-      <c r="I31" s="18" t="n">
-        <v>0.7754</v>
-      </c>
-      <c r="J31" s="18" t="n">
-        <v>0.611</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>COALINDIA</t>
-        </is>
-      </c>
-      <c r="B32" s="18" t="n">
-        <v>19.6727</v>
-      </c>
-      <c r="C32" s="18" t="n">
-        <v>16.8768</v>
-      </c>
-      <c r="D32" s="18" t="n">
-        <v>4.4424</v>
-      </c>
-      <c r="E32" s="18" t="n">
-        <v>95.55759999999999</v>
-      </c>
-      <c r="F32" s="18" t="n">
-        <v>0.7633</v>
-      </c>
-      <c r="G32" s="18" t="n">
-        <v>55.3911</v>
-      </c>
-      <c r="H32" s="18" t="n">
-        <v>0.5395</v>
-      </c>
-      <c r="I32" s="18" t="n">
-        <v>0.8506</v>
-      </c>
-      <c r="J32" s="18" t="n">
-        <v>0.6602</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
-        <is>
-          <t>RELIANCE</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="n">
-        <v>48.5468</v>
-      </c>
-      <c r="C33" s="18" t="n">
-        <v>38.8203</v>
-      </c>
-      <c r="D33" s="18" t="n">
-        <v>2.8866</v>
-      </c>
-      <c r="E33" s="18" t="n">
-        <v>97.1134</v>
-      </c>
-      <c r="F33" s="18" t="n">
-        <v>0.7538</v>
-      </c>
-      <c r="G33" s="18" t="n">
-        <v>51.3742</v>
-      </c>
-      <c r="H33" s="18" t="n">
-        <v>0.5068</v>
-      </c>
-      <c r="I33" s="18" t="n">
-        <v>0.7915</v>
-      </c>
-      <c r="J33" s="18" t="n">
-        <v>0.6179</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="17" t="inlineStr">
-        <is>
-          <t>TITAN</t>
-        </is>
-      </c>
-      <c r="B34" s="18" t="n">
-        <v>200.8666</v>
-      </c>
-      <c r="C34" s="18" t="n">
-        <v>157.9595</v>
-      </c>
-      <c r="D34" s="18" t="n">
-        <v>4.0546</v>
-      </c>
-      <c r="E34" s="18" t="n">
-        <v>95.94540000000001</v>
-      </c>
-      <c r="F34" s="18" t="n">
-        <v>0.7357</v>
-      </c>
-      <c r="G34" s="18" t="n">
-        <v>48.6258</v>
-      </c>
-      <c r="H34" s="18" t="n">
-        <v>0.4717</v>
-      </c>
-      <c r="I34" s="18" t="n">
-        <v>0.1042</v>
-      </c>
-      <c r="J34" s="18" t="n">
-        <v>0.1706</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="B50" s="16" t="n">
+        <v>17.2262</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <v>12.6092</v>
+      </c>
+      <c r="D50" s="16" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="E50" s="16" t="n">
+        <v>99.0005</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <v>0.9297</v>
+      </c>
+      <c r="G50" s="16" t="n">
+        <v>48.583</v>
+      </c>
+      <c r="H50" s="16" t="n">
+        <v>0.4826</v>
+      </c>
+      <c r="I50" s="16" t="n">
+        <v>0.3347</v>
+      </c>
+      <c r="J50" s="16" t="n">
+        <v>0.3952</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>ULTRACEMCO</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n">
-        <v>320.2495</v>
-      </c>
-      <c r="C35" s="18" t="n">
-        <v>250.2662</v>
-      </c>
-      <c r="D35" s="18" t="n">
-        <v>2.1596</v>
-      </c>
-      <c r="E35" s="18" t="n">
-        <v>97.8404</v>
-      </c>
-      <c r="F35" s="18" t="n">
-        <v>0.7205</v>
-      </c>
-      <c r="G35" s="18" t="n">
-        <v>50.5285</v>
-      </c>
-      <c r="H35" s="18" t="n">
-        <v>0.5115</v>
-      </c>
-      <c r="I35" s="18" t="n">
-        <v>0.3739</v>
-      </c>
-      <c r="J35" s="18" t="n">
-        <v>0.432</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B36" s="18" t="n">
-        <v>151.0429</v>
-      </c>
-      <c r="C36" s="18" t="n">
-        <v>117.7514</v>
-      </c>
-      <c r="D36" s="18" t="n">
-        <v>3.1624</v>
-      </c>
-      <c r="E36" s="18" t="n">
-        <v>96.83759999999999</v>
-      </c>
-      <c r="F36" s="18" t="n">
-        <v>0.7194</v>
-      </c>
-      <c r="G36" s="18" t="n">
-        <v>49.8943</v>
-      </c>
-      <c r="H36" s="18" t="n">
-        <v>0.4769</v>
-      </c>
-      <c r="I36" s="18" t="n">
-        <v>0.4079</v>
-      </c>
-      <c r="J36" s="18" t="n">
-        <v>0.4397</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B37" s="20" t="n">
-        <v>17.1126</v>
-      </c>
-      <c r="C37" s="20" t="n">
-        <v>14.8291</v>
-      </c>
-      <c r="D37" s="20" t="n">
-        <v>4.3248</v>
-      </c>
-      <c r="E37" s="20" t="n">
-        <v>95.6752</v>
-      </c>
-      <c r="F37" s="20" t="n">
-        <v>0.6815</v>
-      </c>
-      <c r="G37" s="20" t="n">
-        <v>53.6998</v>
-      </c>
-      <c r="H37" s="20" t="n">
-        <v>0.5285</v>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v>0.7046</v>
-      </c>
-      <c r="J37" s="20" t="n">
-        <v>0.604</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>BPCL</t>
-        </is>
-      </c>
-      <c r="B38" s="20" t="n">
-        <v>20.6124</v>
-      </c>
-      <c r="C38" s="20" t="n">
-        <v>15.9742</v>
-      </c>
-      <c r="D38" s="20" t="n">
-        <v>4.9007</v>
-      </c>
-      <c r="E38" s="20" t="n">
-        <v>95.0993</v>
-      </c>
-      <c r="F38" s="20" t="n">
-        <v>0.6625</v>
-      </c>
-      <c r="G38" s="20" t="n">
-        <v>53.9112</v>
-      </c>
-      <c r="H38" s="20" t="n">
-        <v>0.5714</v>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v>0.1416</v>
-      </c>
-      <c r="J38" s="20" t="n">
-        <v>0.227</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n">
-        <v>48.3634</v>
-      </c>
-      <c r="C39" s="20" t="n">
-        <v>38.0968</v>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>2.1681</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <v>97.8319</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>0.6521</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>50.9514</v>
-      </c>
-      <c r="H39" s="20" t="n">
-        <v>0.5893</v>
-      </c>
-      <c r="I39" s="20" t="n">
-        <v>0.2619</v>
-      </c>
-      <c r="J39" s="20" t="n">
-        <v>0.3626</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="19" t="inlineStr">
-        <is>
-          <t>APOLLOHOSP</t>
-        </is>
-      </c>
-      <c r="B40" s="20" t="n">
-        <v>323.0114</v>
-      </c>
-      <c r="C40" s="20" t="n">
-        <v>255.7491</v>
-      </c>
-      <c r="D40" s="20" t="n">
-        <v>3.3879</v>
-      </c>
-      <c r="E40" s="20" t="n">
-        <v>96.6121</v>
-      </c>
-      <c r="F40" s="20" t="n">
-        <v>0.6354</v>
-      </c>
-      <c r="G40" s="20" t="n">
-        <v>51.3742</v>
-      </c>
-      <c r="H40" s="20" t="n">
-        <v>0.5238</v>
-      </c>
-      <c r="I40" s="20" t="n">
-        <v>0.1416</v>
-      </c>
-      <c r="J40" s="20" t="n">
-        <v>0.223</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B41" s="20" t="n">
-        <v>617.564</v>
-      </c>
-      <c r="C41" s="20" t="n">
-        <v>475.4049</v>
-      </c>
-      <c r="D41" s="20" t="n">
-        <v>5.2498</v>
-      </c>
-      <c r="E41" s="20" t="n">
-        <v>94.75020000000001</v>
-      </c>
-      <c r="F41" s="20" t="n">
-        <v>0.6054</v>
-      </c>
-      <c r="G41" s="20" t="n">
-        <v>50.74</v>
-      </c>
-      <c r="H41" s="20" t="n">
-        <v>0.5183</v>
-      </c>
-      <c r="I41" s="20" t="n">
-        <v>0.6393</v>
-      </c>
-      <c r="J41" s="20" t="n">
-        <v>0.5725</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="19" t="inlineStr">
-        <is>
-          <t>SHRIRAMFIN</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="n">
-        <v>110.139</v>
-      </c>
-      <c r="C42" s="20" t="n">
-        <v>75.53570000000001</v>
-      </c>
-      <c r="D42" s="20" t="n">
-        <v>8.555400000000001</v>
-      </c>
-      <c r="E42" s="20" t="n">
-        <v>91.44459999999999</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>0.5809</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>51.5856</v>
-      </c>
-      <c r="H42" s="20" t="n">
-        <v>0.5844</v>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="J42" s="20" t="n">
-        <v>0.2821</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="19" t="inlineStr">
-        <is>
-          <t>M&amp;M</t>
-        </is>
-      </c>
-      <c r="B43" s="20" t="n">
-        <v>205.0387</v>
-      </c>
-      <c r="C43" s="20" t="n">
-        <v>163.6477</v>
-      </c>
-      <c r="D43" s="20" t="n">
-        <v>4.9995</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>95.0005</v>
-      </c>
-      <c r="F43" s="20" t="n">
-        <v>0.5706</v>
-      </c>
-      <c r="G43" s="20" t="n">
-        <v>52.0085</v>
-      </c>
-      <c r="H43" s="20" t="n">
-        <v>0.5728</v>
-      </c>
-      <c r="I43" s="20" t="n">
-        <v>0.2438</v>
-      </c>
-      <c r="J43" s="20" t="n">
-        <v>0.342</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>BAJAJFINSV</t>
-        </is>
-      </c>
-      <c r="B44" s="20" t="n">
-        <v>100.6795</v>
-      </c>
-      <c r="C44" s="20" t="n">
-        <v>84.70740000000001</v>
-      </c>
-      <c r="D44" s="20" t="n">
-        <v>4.3436</v>
-      </c>
-      <c r="E44" s="20" t="n">
-        <v>95.6564</v>
-      </c>
-      <c r="F44" s="20" t="n">
-        <v>0.5679999999999999</v>
-      </c>
-      <c r="G44" s="20" t="n">
-        <v>50.74</v>
-      </c>
-      <c r="H44" s="20" t="n">
-        <v>0.527</v>
-      </c>
-      <c r="I44" s="20" t="n">
-        <v>0.1646</v>
-      </c>
-      <c r="J44" s="20" t="n">
-        <v>0.2508</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="19" t="inlineStr">
-        <is>
-          <t>EICHERMOT</t>
-        </is>
-      </c>
-      <c r="B45" s="20" t="n">
-        <v>787.3495</v>
-      </c>
-      <c r="C45" s="20" t="n">
-        <v>603.4223</v>
-      </c>
-      <c r="D45" s="20" t="n">
-        <v>8.875999999999999</v>
-      </c>
-      <c r="E45" s="20" t="n">
-        <v>91.124</v>
-      </c>
-      <c r="F45" s="20" t="n">
-        <v>0.4656</v>
-      </c>
-      <c r="G45" s="20" t="n">
-        <v>49.26</v>
-      </c>
-      <c r="H45" s="20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v>0.0458</v>
-      </c>
-      <c r="J45" s="20" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="19" t="inlineStr">
-        <is>
-          <t>BAJFINANCE</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="n">
-        <v>85.372</v>
-      </c>
-      <c r="C46" s="20" t="n">
-        <v>70.77930000000001</v>
-      </c>
-      <c r="D46" s="20" t="n">
-        <v>7.5679</v>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>92.43210000000001</v>
-      </c>
-      <c r="F46" s="20" t="n">
-        <v>0.4593</v>
-      </c>
-      <c r="G46" s="20" t="n">
-        <v>48.8372</v>
-      </c>
-      <c r="H46" s="20" t="n">
-        <v>0.5780999999999999</v>
-      </c>
-      <c r="I46" s="20" t="n">
-        <v>0.1468</v>
-      </c>
-      <c r="J46" s="20" t="n">
-        <v>0.2342</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="19" t="inlineStr">
-        <is>
-          <t>JSWSTEEL</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
-        <v>88.7216</v>
-      </c>
-      <c r="C47" s="20" t="n">
-        <v>76.4573</v>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>6.8068</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>93.1932</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0.4291</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>47.1459</v>
-      </c>
-      <c r="H47" s="20" t="n">
-        <v>0.4615</v>
-      </c>
-      <c r="I47" s="20" t="n">
-        <v>0.0241</v>
-      </c>
-      <c r="J47" s="20" t="n">
-        <v>0.0458</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
-        <is>
-          <t>POWERGRID</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
-        <v>14.8611</v>
-      </c>
-      <c r="C48" s="20" t="n">
-        <v>13.232</v>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4.7029</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>95.2971</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0.4209</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>49.8943</v>
-      </c>
-      <c r="H48" s="20" t="n">
-        <v>0.4966</v>
-      </c>
-      <c r="I48" s="20" t="n">
-        <v>0.9359</v>
-      </c>
-      <c r="J48" s="20" t="n">
-        <v>0.6489</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>ICICIBANK</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
-        <v>70.89709999999999</v>
-      </c>
-      <c r="C49" s="20" t="n">
-        <v>61.5725</v>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>4.5078</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>95.4922</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>0.1836</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>50.74</v>
-      </c>
-      <c r="H49" s="20" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="I49" s="20" t="n">
-        <v>0.0498</v>
-      </c>
-      <c r="J49" s="20" t="n">
-        <v>0.0934</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="19" t="inlineStr">
-        <is>
-          <t>DIVISLAB</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n">
-        <v>426.5868</v>
-      </c>
-      <c r="C50" s="20" t="n">
-        <v>374.6763</v>
-      </c>
-      <c r="D50" s="20" t="n">
-        <v>5.9379</v>
-      </c>
-      <c r="E50" s="20" t="n">
-        <v>94.0621</v>
-      </c>
-      <c r="F50" s="20" t="n">
-        <v>0.1804</v>
-      </c>
-      <c r="G50" s="20" t="n">
-        <v>49.0486</v>
-      </c>
-      <c r="H50" s="20" t="n">
-        <v>0.6471</v>
-      </c>
-      <c r="I50" s="20" t="n">
-        <v>0.0447</v>
-      </c>
-      <c r="J50" s="20" t="n">
-        <v>0.0837</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="21" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B51" s="22" t="n">
-        <v>243.5228</v>
-      </c>
-      <c r="C51" s="22" t="n">
-        <v>208.2696</v>
-      </c>
-      <c r="D51" s="22" t="n">
-        <v>10.8948</v>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>89.1052</v>
-      </c>
-      <c r="F51" s="22" t="n">
-        <v>-0.9275</v>
-      </c>
-      <c r="G51" s="22" t="n">
-        <v>47.9915</v>
-      </c>
-      <c r="H51" s="22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I51" s="22" t="n">
-        <v>0.0325</v>
-      </c>
-      <c r="J51" s="22" t="n">
-        <v>0.0611</v>
+      <c r="B51" s="16" t="n">
+        <v>164.1219</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <v>121.7957</v>
+      </c>
+      <c r="D51" s="16" t="n">
+        <v>1.055</v>
+      </c>
+      <c r="E51" s="16" t="n">
+        <v>98.94499999999999</v>
+      </c>
+      <c r="F51" s="16" t="n">
+        <v>0.924</v>
+      </c>
+      <c r="G51" s="16" t="n">
+        <v>48.1781</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>0.4872</v>
+      </c>
+      <c r="I51" s="16" t="n">
+        <v>0.9385</v>
+      </c>
+      <c r="J51" s="16" t="n">
+        <v>0.6415</v>
       </c>
     </row>
   </sheetData>
@@ -14202,206 +14169,206 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>ARIMA</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="18" t="n">
         <v>311.4102</v>
       </c>
-      <c r="C2" s="24" t="n">
+      <c r="C2" s="18" t="n">
         <v>260.3912</v>
       </c>
-      <c r="D2" s="24" t="n">
+      <c r="D2" s="18" t="n">
         <v>11.0469</v>
       </c>
-      <c r="E2" s="24" t="n">
+      <c r="E2" s="18" t="n">
         <v>88.95310000000001</v>
       </c>
-      <c r="F2" s="24" t="n">
+      <c r="F2" s="18" t="n">
         <v>-1.1632</v>
       </c>
-      <c r="G2" s="24" t="n">
+      <c r="G2" s="18" t="n">
         <v>50.75</v>
       </c>
-      <c r="H2" s="24" t="n">
+      <c r="H2" s="18" t="n">
         <v>0.5347</v>
       </c>
-      <c r="I2" s="24" t="n">
+      <c r="I2" s="18" t="n">
         <v>0.5118</v>
       </c>
-      <c r="J2" s="24" t="n">
+      <c r="J2" s="18" t="n">
         <v>0.4502</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>SARIMA</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="18" t="n">
         <v>310.641</v>
       </c>
-      <c r="C3" s="24" t="n">
+      <c r="C3" s="18" t="n">
         <v>259.8228</v>
       </c>
-      <c r="D3" s="24" t="n">
+      <c r="D3" s="18" t="n">
         <v>11.0606</v>
       </c>
-      <c r="E3" s="24" t="n">
+      <c r="E3" s="18" t="n">
         <v>88.93940000000001</v>
       </c>
-      <c r="F3" s="24" t="n">
+      <c r="F3" s="18" t="n">
         <v>-1.1649</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="G3" s="18" t="n">
         <v>50.7097</v>
       </c>
-      <c r="H3" s="24" t="n">
+      <c r="H3" s="18" t="n">
         <v>0.5365</v>
       </c>
-      <c r="I3" s="24" t="n">
+      <c r="I3" s="18" t="n">
         <v>0.5118</v>
       </c>
-      <c r="J3" s="24" t="n">
+      <c r="J3" s="18" t="n">
         <v>0.4495</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>ARIMA-LSTM</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="18" t="n">
         <v>38.4275</v>
       </c>
-      <c r="C4" s="24" t="n">
+      <c r="C4" s="18" t="n">
         <v>27.5468</v>
       </c>
-      <c r="D4" s="24" t="n">
+      <c r="D4" s="18" t="n">
         <v>1.1398</v>
       </c>
-      <c r="E4" s="24" t="n">
+      <c r="E4" s="18" t="n">
         <v>98.86020000000001</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="18" t="n">
         <v>0.9736</v>
       </c>
-      <c r="G4" s="24" t="n">
+      <c r="G4" s="18" t="n">
         <v>50.063</v>
       </c>
-      <c r="H4" s="24" t="n">
+      <c r="H4" s="18" t="n">
         <v>0.4947</v>
       </c>
-      <c r="I4" s="24" t="n">
+      <c r="I4" s="18" t="n">
         <v>0.6133</v>
       </c>
-      <c r="J4" s="24" t="n">
+      <c r="J4" s="18" t="n">
         <v>0.4805</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="18" t="n">
         <v>264.1898</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="18" t="n">
         <v>206.261</v>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="18" t="n">
         <v>7.3715</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="18" t="n">
         <v>92.6285</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="18" t="n">
         <v>-0.2332</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="G5" s="18" t="n">
         <v>51.0831</v>
       </c>
-      <c r="H5" s="24" t="n">
+      <c r="H5" s="18" t="n">
         <v>0.5361</v>
       </c>
-      <c r="I5" s="24" t="n">
+      <c r="I5" s="18" t="n">
         <v>0.3787</v>
       </c>
-      <c r="J5" s="24" t="n">
+      <c r="J5" s="18" t="n">
         <v>0.3719</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>LSTM</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="18" t="n">
         <v>120.3097</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="18" t="n">
         <v>94.33839999999999</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="18" t="n">
         <v>3.756</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="18" t="n">
         <v>96.244</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="18" t="n">
         <v>0.7229</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="18" t="n">
         <v>50.8153</v>
       </c>
-      <c r="H6" s="24" t="n">
+      <c r="H6" s="18" t="n">
         <v>0.5131</v>
       </c>
-      <c r="I6" s="24" t="n">
+      <c r="I6" s="18" t="n">
         <v>0.3542</v>
       </c>
-      <c r="J6" s="24" t="n">
+      <c r="J6" s="18" t="n">
         <v>0.362</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>CNN-LSTM</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="20" t="n">
         <v>126.5844</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="20" t="n">
         <v>99.3085</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="20" t="n">
         <v>3.7932</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="20" t="n">
         <v>96.2068</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="20" t="n">
         <v>0.7252999999999999</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="20" t="n">
         <v>50.7291</v>
       </c>
-      <c r="H7" s="26" t="n">
+      <c r="H7" s="20" t="n">
         <v>0.5236</v>
       </c>
-      <c r="I7" s="26" t="n">
+      <c r="I7" s="20" t="n">
         <v>0.3941</v>
       </c>
-      <c r="J7" s="26" t="n">
+      <c r="J7" s="20" t="n">
         <v>0.3952</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model order in charts and excel to ARIMA, SARIMA, XGBoost, LSTM, CNN-LSTM, ARIMA-LSTM
</commit_message>
<xml_diff>
--- a/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
+++ b/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
@@ -14239,137 +14239,137 @@
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>ARIMA-LSTM</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>38.4275</v>
+        <v>264.1898</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>27.5468</v>
+        <v>206.261</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>1.1398</v>
+        <v>7.3715</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>98.86020000000001</v>
+        <v>92.6285</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>0.9736</v>
+        <v>-0.2332</v>
       </c>
       <c r="G4" s="18" t="n">
-        <v>50.063</v>
+        <v>51.0831</v>
       </c>
       <c r="H4" s="18" t="n">
-        <v>0.4947</v>
+        <v>0.5361</v>
       </c>
       <c r="I4" s="18" t="n">
-        <v>0.6133</v>
+        <v>0.3787</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>0.4805</v>
+        <v>0.3719</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>264.1898</v>
+        <v>120.3097</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>206.261</v>
+        <v>94.33839999999999</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>7.3715</v>
+        <v>3.756</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>92.6285</v>
+        <v>96.244</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>-0.2332</v>
+        <v>0.7229</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>51.0831</v>
+        <v>50.8153</v>
       </c>
       <c r="H5" s="18" t="n">
-        <v>0.5361</v>
+        <v>0.5131</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>0.3787</v>
+        <v>0.3542</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.3719</v>
+        <v>0.362</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>LSTM</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="n">
-        <v>120.3097</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>94.33839999999999</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>3.756</v>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>96.244</v>
-      </c>
-      <c r="F6" s="18" t="n">
-        <v>0.7229</v>
-      </c>
-      <c r="G6" s="18" t="n">
-        <v>50.8153</v>
-      </c>
-      <c r="H6" s="18" t="n">
-        <v>0.5131</v>
-      </c>
-      <c r="I6" s="18" t="n">
-        <v>0.3542</v>
-      </c>
-      <c r="J6" s="18" t="n">
-        <v>0.362</v>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>CNN-LSTM</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>126.5844</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>99.3085</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>3.7932</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>96.2068</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>0.7252999999999999</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>50.7291</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>0.5236</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>0.3941</v>
+      </c>
+      <c r="J6" s="20" t="n">
+        <v>0.3952</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>CNN-LSTM</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>126.5844</v>
-      </c>
-      <c r="C7" s="20" t="n">
-        <v>99.3085</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <v>3.7932</v>
-      </c>
-      <c r="E7" s="20" t="n">
-        <v>96.2068</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>0.7252999999999999</v>
-      </c>
-      <c r="G7" s="20" t="n">
-        <v>50.7291</v>
-      </c>
-      <c r="H7" s="20" t="n">
-        <v>0.5236</v>
-      </c>
-      <c r="I7" s="20" t="n">
-        <v>0.3941</v>
-      </c>
-      <c r="J7" s="20" t="n">
-        <v>0.3952</v>
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>ARIMA-LSTM</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>38.4275</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>27.5468</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>1.1398</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>98.86020000000001</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>0.9736</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>50.063</v>
+      </c>
+      <c r="H7" s="18" t="n">
+        <v>0.4947</v>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>0.6133</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <v>0.4805</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix graph text labels to say ARIMA-LSTM instead of CNN-LSTM
</commit_message>
<xml_diff>
--- a/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
+++ b/backend/ml_service/dissertation_results/report/dissertation_table.xlsx
@@ -66,12 +66,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4D0A0"/>
+        <fgColor rgb="002E8B57"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E8B57"/>
+        <fgColor rgb="0032CD32"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,16 +123,16 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -153,7 +153,7 @@
     <xf numFmtId="164" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -14305,70 +14305,70 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>CNN-LSTM</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
+      <c r="B6" s="18" t="n">
         <v>126.5844</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="18" t="n">
         <v>99.3085</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="18" t="n">
         <v>3.7932</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="18" t="n">
         <v>96.2068</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="18" t="n">
         <v>0.7252999999999999</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="18" t="n">
         <v>50.7291</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="18" t="n">
         <v>0.5236</v>
       </c>
-      <c r="I6" s="20" t="n">
+      <c r="I6" s="18" t="n">
         <v>0.3941</v>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="J6" s="18" t="n">
         <v>0.3952</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>ARIMA-LSTM</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="20" t="n">
         <v>38.4275</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="20" t="n">
         <v>27.5468</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="20" t="n">
         <v>1.1398</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="20" t="n">
         <v>98.86020000000001</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="20" t="n">
         <v>0.9736</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="20" t="n">
         <v>50.063</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="20" t="n">
         <v>0.4947</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="20" t="n">
         <v>0.6133</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="20" t="n">
         <v>0.4805</v>
       </c>
     </row>

</xml_diff>